<commit_message>
Time series correction to new files
</commit_message>
<xml_diff>
--- a/InputData/elec/BCpUC/Battery Cost per Unit Cap.xlsx
+++ b/InputData/elec/BCpUC/Battery Cost per Unit Cap.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energyinnovation-my.sharepoint.com/personal/maryfrancis_energyinnovation_org/Documents/South Korea/4.0.5/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\elec\BCpUC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{935069C4-DFE3-4F75-8831-FDBCBA4C7C33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2958B585-FE57-483E-889A-B3CF2BDE2F44}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD84EB8-A062-4DE5-9603-10309A2960B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27975" yWindow="-360" windowWidth="23625" windowHeight="15345" tabRatio="839" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="839" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Claude Log" sheetId="14" r:id="rId1"/>
@@ -2138,7 +2138,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="233">
+  <cellXfs count="232">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2536,83 +2536,32 @@
     <xf numFmtId="173" fontId="1" fillId="0" borderId="78" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="23" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="28" fillId="22" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -2659,6 +2608,60 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2668,10 +2671,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Body: normal cell" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -5630,37 +5629,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="36" customHeight="1">
-      <c r="A1" s="179" t="s">
+      <c r="A1" s="183" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="180"/>
-      <c r="C1" s="180"/>
-      <c r="D1" s="180"/>
-      <c r="E1" s="180"/>
-      <c r="F1" s="180"/>
-      <c r="G1" s="180"/>
-      <c r="H1" s="180"/>
-      <c r="I1" s="180"/>
-      <c r="J1" s="180"/>
-      <c r="K1" s="180"/>
-      <c r="L1" s="180"/>
+      <c r="B1" s="181"/>
+      <c r="C1" s="181"/>
+      <c r="D1" s="181"/>
+      <c r="E1" s="181"/>
+      <c r="F1" s="181"/>
+      <c r="G1" s="181"/>
+      <c r="H1" s="181"/>
+      <c r="I1" s="181"/>
+      <c r="J1" s="181"/>
+      <c r="K1" s="181"/>
+      <c r="L1" s="181"/>
     </row>
     <row r="2" spans="1:12" ht="30" customHeight="1"/>
     <row r="3" spans="1:12" ht="24" customHeight="1">
-      <c r="A3" s="181" t="s">
+      <c r="A3" s="180" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="180"/>
-      <c r="C3" s="180"/>
-      <c r="D3" s="180"/>
-      <c r="E3" s="180"/>
-      <c r="F3" s="180"/>
-      <c r="G3" s="180"/>
-      <c r="H3" s="180"/>
-      <c r="I3" s="180"/>
-      <c r="J3" s="180"/>
-      <c r="K3" s="180"/>
-      <c r="L3" s="180"/>
+      <c r="B3" s="181"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
+      <c r="H3" s="181"/>
+      <c r="I3" s="181"/>
+      <c r="J3" s="181"/>
+      <c r="K3" s="181"/>
+      <c r="L3" s="181"/>
     </row>
     <row r="4" spans="1:12" ht="20.149999999999999" customHeight="1">
       <c r="A4" s="148" t="s">
@@ -5750,20 +5749,20 @@
     </row>
     <row r="9" spans="1:12" ht="20.149999999999999" customHeight="1"/>
     <row r="10" spans="1:12" ht="20.149999999999999" customHeight="1">
-      <c r="A10" s="181" t="s">
+      <c r="A10" s="180" t="s">
         <v>187</v>
       </c>
-      <c r="B10" s="183"/>
-      <c r="C10" s="183"/>
-      <c r="D10" s="183"/>
-      <c r="E10" s="183"/>
-      <c r="F10" s="183"/>
-      <c r="G10" s="183"/>
-      <c r="H10" s="183"/>
-      <c r="I10" s="183"/>
-      <c r="J10" s="183"/>
-      <c r="K10" s="183"/>
-      <c r="L10" s="183"/>
+      <c r="B10" s="184"/>
+      <c r="C10" s="184"/>
+      <c r="D10" s="184"/>
+      <c r="E10" s="184"/>
+      <c r="F10" s="184"/>
+      <c r="G10" s="184"/>
+      <c r="H10" s="184"/>
+      <c r="I10" s="184"/>
+      <c r="J10" s="184"/>
+      <c r="K10" s="184"/>
+      <c r="L10" s="184"/>
     </row>
     <row r="11" spans="1:12" ht="20.149999999999999" customHeight="1">
       <c r="A11" s="149" t="s">
@@ -5949,32 +5948,32 @@
       </c>
     </row>
     <row r="21" spans="1:12" ht="24" customHeight="1">
-      <c r="A21" s="181" t="s">
+      <c r="A21" s="180" t="s">
         <v>193</v>
       </c>
-      <c r="B21" s="180"/>
-      <c r="C21" s="180"/>
-      <c r="D21" s="180"/>
-      <c r="E21" s="180"/>
-      <c r="F21" s="180"/>
-      <c r="G21" s="180"/>
-      <c r="H21" s="180"/>
-      <c r="I21" s="180"/>
-      <c r="J21" s="180"/>
-      <c r="K21" s="180"/>
-      <c r="L21" s="180"/>
+      <c r="B21" s="181"/>
+      <c r="C21" s="181"/>
+      <c r="D21" s="181"/>
+      <c r="E21" s="181"/>
+      <c r="F21" s="181"/>
+      <c r="G21" s="181"/>
+      <c r="H21" s="181"/>
+      <c r="I21" s="181"/>
+      <c r="J21" s="181"/>
+      <c r="K21" s="181"/>
+      <c r="L21" s="181"/>
     </row>
     <row r="22" spans="1:12" ht="18" customHeight="1">
       <c r="A22" s="182" t="s">
         <v>194</v>
       </c>
-      <c r="B22" s="180"/>
-      <c r="C22" s="180"/>
-      <c r="D22" s="180"/>
-      <c r="E22" s="180"/>
-      <c r="F22" s="180"/>
-      <c r="G22" s="180"/>
-      <c r="H22" s="180"/>
+      <c r="B22" s="181"/>
+      <c r="C22" s="181"/>
+      <c r="D22" s="181"/>
+      <c r="E22" s="181"/>
+      <c r="F22" s="181"/>
+      <c r="G22" s="181"/>
+      <c r="H22" s="181"/>
     </row>
     <row r="23" spans="1:12" ht="20.149999999999999" customHeight="1">
       <c r="A23" s="149" t="s">
@@ -6212,32 +6211,32 @@
     </row>
     <row r="32" spans="1:12" ht="20.149999999999999" customHeight="1"/>
     <row r="33" spans="1:33" ht="20.149999999999999" customHeight="1">
-      <c r="A33" s="181" t="s">
+      <c r="A33" s="180" t="s">
         <v>201</v>
       </c>
-      <c r="B33" s="180"/>
-      <c r="C33" s="180"/>
-      <c r="D33" s="180"/>
-      <c r="E33" s="180"/>
-      <c r="F33" s="180"/>
-      <c r="G33" s="180"/>
-      <c r="H33" s="180"/>
-      <c r="I33" s="180"/>
-      <c r="J33" s="180"/>
-      <c r="K33" s="180"/>
-      <c r="L33" s="180"/>
+      <c r="B33" s="181"/>
+      <c r="C33" s="181"/>
+      <c r="D33" s="181"/>
+      <c r="E33" s="181"/>
+      <c r="F33" s="181"/>
+      <c r="G33" s="181"/>
+      <c r="H33" s="181"/>
+      <c r="I33" s="181"/>
+      <c r="J33" s="181"/>
+      <c r="K33" s="181"/>
+      <c r="L33" s="181"/>
     </row>
     <row r="34" spans="1:33" ht="18" customHeight="1">
-      <c r="A34" s="184" t="s">
+      <c r="A34" s="185" t="s">
         <v>202</v>
       </c>
-      <c r="B34" s="180"/>
-      <c r="C34" s="180"/>
-      <c r="D34" s="180"/>
-      <c r="E34" s="180"/>
-      <c r="F34" s="180"/>
-      <c r="G34" s="180"/>
-      <c r="H34" s="180"/>
+      <c r="B34" s="181"/>
+      <c r="C34" s="181"/>
+      <c r="D34" s="181"/>
+      <c r="E34" s="181"/>
+      <c r="F34" s="181"/>
+      <c r="G34" s="181"/>
+      <c r="H34" s="181"/>
     </row>
     <row r="35" spans="1:33" ht="20.149999999999999" customHeight="1">
       <c r="A35" s="149" t="s">
@@ -6460,78 +6459,78 @@
       <c r="H44" s="159"/>
     </row>
     <row r="45" spans="1:33" ht="24" customHeight="1">
-      <c r="A45" s="181" t="s">
+      <c r="A45" s="180" t="s">
         <v>208</v>
       </c>
-      <c r="B45" s="180"/>
-      <c r="C45" s="180"/>
-      <c r="D45" s="180"/>
-      <c r="E45" s="180"/>
-      <c r="F45" s="180"/>
-      <c r="G45" s="180"/>
-      <c r="H45" s="180"/>
-      <c r="I45" s="180"/>
-      <c r="J45" s="180"/>
-      <c r="K45" s="180"/>
-      <c r="L45" s="180"/>
-      <c r="M45" s="180"/>
-      <c r="N45" s="180"/>
-      <c r="O45" s="180"/>
-      <c r="P45" s="180"/>
-      <c r="Q45" s="180"/>
-      <c r="R45" s="180"/>
-      <c r="S45" s="180"/>
-      <c r="T45" s="180"/>
-      <c r="U45" s="180"/>
-      <c r="V45" s="180"/>
-      <c r="W45" s="180"/>
-      <c r="X45" s="180"/>
-      <c r="Y45" s="180"/>
-      <c r="Z45" s="180"/>
-      <c r="AA45" s="180"/>
-      <c r="AB45" s="180"/>
-      <c r="AC45" s="180"/>
-      <c r="AD45" s="180"/>
-      <c r="AE45" s="180"/>
-      <c r="AF45" s="180"/>
-      <c r="AG45" s="180"/>
+      <c r="B45" s="181"/>
+      <c r="C45" s="181"/>
+      <c r="D45" s="181"/>
+      <c r="E45" s="181"/>
+      <c r="F45" s="181"/>
+      <c r="G45" s="181"/>
+      <c r="H45" s="181"/>
+      <c r="I45" s="181"/>
+      <c r="J45" s="181"/>
+      <c r="K45" s="181"/>
+      <c r="L45" s="181"/>
+      <c r="M45" s="181"/>
+      <c r="N45" s="181"/>
+      <c r="O45" s="181"/>
+      <c r="P45" s="181"/>
+      <c r="Q45" s="181"/>
+      <c r="R45" s="181"/>
+      <c r="S45" s="181"/>
+      <c r="T45" s="181"/>
+      <c r="U45" s="181"/>
+      <c r="V45" s="181"/>
+      <c r="W45" s="181"/>
+      <c r="X45" s="181"/>
+      <c r="Y45" s="181"/>
+      <c r="Z45" s="181"/>
+      <c r="AA45" s="181"/>
+      <c r="AB45" s="181"/>
+      <c r="AC45" s="181"/>
+      <c r="AD45" s="181"/>
+      <c r="AE45" s="181"/>
+      <c r="AF45" s="181"/>
+      <c r="AG45" s="181"/>
     </row>
     <row r="46" spans="1:33" ht="20.149999999999999" customHeight="1">
       <c r="A46" s="182" t="s">
         <v>210</v>
       </c>
-      <c r="B46" s="180"/>
-      <c r="C46" s="180"/>
-      <c r="D46" s="180"/>
-      <c r="E46" s="180"/>
-      <c r="F46" s="180"/>
-      <c r="G46" s="180"/>
-      <c r="H46" s="180"/>
-      <c r="I46" s="180"/>
-      <c r="J46" s="180"/>
-      <c r="K46" s="180"/>
-      <c r="L46" s="180"/>
-      <c r="M46" s="180"/>
-      <c r="N46" s="180"/>
-      <c r="O46" s="180"/>
-      <c r="P46" s="180"/>
-      <c r="Q46" s="180"/>
-      <c r="R46" s="180"/>
-      <c r="S46" s="180"/>
-      <c r="T46" s="180"/>
-      <c r="U46" s="180"/>
-      <c r="V46" s="180"/>
-      <c r="W46" s="180"/>
-      <c r="X46" s="180"/>
-      <c r="Y46" s="180"/>
-      <c r="Z46" s="180"/>
-      <c r="AA46" s="180"/>
-      <c r="AB46" s="180"/>
-      <c r="AC46" s="180"/>
-      <c r="AD46" s="180"/>
-      <c r="AE46" s="180"/>
-      <c r="AF46" s="180"/>
-      <c r="AG46" s="180"/>
+      <c r="B46" s="181"/>
+      <c r="C46" s="181"/>
+      <c r="D46" s="181"/>
+      <c r="E46" s="181"/>
+      <c r="F46" s="181"/>
+      <c r="G46" s="181"/>
+      <c r="H46" s="181"/>
+      <c r="I46" s="181"/>
+      <c r="J46" s="181"/>
+      <c r="K46" s="181"/>
+      <c r="L46" s="181"/>
+      <c r="M46" s="181"/>
+      <c r="N46" s="181"/>
+      <c r="O46" s="181"/>
+      <c r="P46" s="181"/>
+      <c r="Q46" s="181"/>
+      <c r="R46" s="181"/>
+      <c r="S46" s="181"/>
+      <c r="T46" s="181"/>
+      <c r="U46" s="181"/>
+      <c r="V46" s="181"/>
+      <c r="W46" s="181"/>
+      <c r="X46" s="181"/>
+      <c r="Y46" s="181"/>
+      <c r="Z46" s="181"/>
+      <c r="AA46" s="181"/>
+      <c r="AB46" s="181"/>
+      <c r="AC46" s="181"/>
+      <c r="AD46" s="181"/>
+      <c r="AE46" s="181"/>
+      <c r="AF46" s="181"/>
+      <c r="AG46" s="181"/>
     </row>
     <row r="47" spans="1:33" ht="22" customHeight="1">
       <c r="A47" s="149" t="s">
@@ -6902,41 +6901,41 @@
       <c r="AJ49"/>
     </row>
     <row r="50" spans="1:36" ht="18" customHeight="1">
-      <c r="A50" s="185" t="s">
+      <c r="A50" s="186" t="s">
         <v>209</v>
       </c>
-      <c r="B50" s="186"/>
-      <c r="C50" s="186"/>
-      <c r="D50" s="186"/>
-      <c r="E50" s="186"/>
-      <c r="F50" s="186"/>
-      <c r="G50" s="186"/>
-      <c r="H50" s="186"/>
-      <c r="I50" s="186"/>
-      <c r="J50" s="186"/>
-      <c r="K50" s="186"/>
-      <c r="L50" s="186"/>
-      <c r="M50" s="186"/>
-      <c r="N50" s="186"/>
-      <c r="O50" s="186"/>
-      <c r="P50" s="186"/>
-      <c r="Q50" s="186"/>
-      <c r="R50" s="186"/>
-      <c r="S50" s="186"/>
-      <c r="T50" s="186"/>
-      <c r="U50" s="186"/>
-      <c r="V50" s="186"/>
-      <c r="W50" s="186"/>
-      <c r="X50" s="186"/>
-      <c r="Y50" s="186"/>
-      <c r="Z50" s="186"/>
-      <c r="AA50" s="186"/>
-      <c r="AB50" s="186"/>
-      <c r="AC50" s="186"/>
-      <c r="AD50" s="186"/>
-      <c r="AE50" s="186"/>
-      <c r="AF50" s="186"/>
-      <c r="AG50" s="186"/>
+      <c r="B50" s="187"/>
+      <c r="C50" s="187"/>
+      <c r="D50" s="187"/>
+      <c r="E50" s="187"/>
+      <c r="F50" s="187"/>
+      <c r="G50" s="187"/>
+      <c r="H50" s="187"/>
+      <c r="I50" s="187"/>
+      <c r="J50" s="187"/>
+      <c r="K50" s="187"/>
+      <c r="L50" s="187"/>
+      <c r="M50" s="187"/>
+      <c r="N50" s="187"/>
+      <c r="O50" s="187"/>
+      <c r="P50" s="187"/>
+      <c r="Q50" s="187"/>
+      <c r="R50" s="187"/>
+      <c r="S50" s="187"/>
+      <c r="T50" s="187"/>
+      <c r="U50" s="187"/>
+      <c r="V50" s="187"/>
+      <c r="W50" s="187"/>
+      <c r="X50" s="187"/>
+      <c r="Y50" s="187"/>
+      <c r="Z50" s="187"/>
+      <c r="AA50" s="187"/>
+      <c r="AB50" s="187"/>
+      <c r="AC50" s="187"/>
+      <c r="AD50" s="187"/>
+      <c r="AE50" s="187"/>
+      <c r="AF50" s="187"/>
+      <c r="AG50" s="187"/>
     </row>
     <row r="51" spans="1:36" ht="18" customHeight="1">
       <c r="A51" s="173" t="s">
@@ -6947,78 +6946,78 @@
       <c r="A52" s="173"/>
     </row>
     <row r="53" spans="1:36" ht="18" customHeight="1">
-      <c r="A53" s="181" t="s">
+      <c r="A53" s="180" t="s">
         <v>234</v>
       </c>
-      <c r="B53" s="180"/>
-      <c r="C53" s="180"/>
-      <c r="D53" s="180"/>
-      <c r="E53" s="180"/>
-      <c r="F53" s="180"/>
-      <c r="G53" s="180"/>
-      <c r="H53" s="180"/>
-      <c r="I53" s="180"/>
-      <c r="J53" s="180"/>
-      <c r="K53" s="180"/>
-      <c r="L53" s="180"/>
-      <c r="M53" s="180"/>
-      <c r="N53" s="180"/>
-      <c r="O53" s="180"/>
-      <c r="P53" s="180"/>
-      <c r="Q53" s="180"/>
-      <c r="R53" s="180"/>
-      <c r="S53" s="180"/>
-      <c r="T53" s="180"/>
-      <c r="U53" s="180"/>
-      <c r="V53" s="180"/>
-      <c r="W53" s="180"/>
-      <c r="X53" s="180"/>
-      <c r="Y53" s="180"/>
-      <c r="Z53" s="180"/>
-      <c r="AA53" s="180"/>
-      <c r="AB53" s="180"/>
-      <c r="AC53" s="180"/>
-      <c r="AD53" s="180"/>
-      <c r="AE53" s="180"/>
-      <c r="AF53" s="180"/>
-      <c r="AG53" s="180"/>
+      <c r="B53" s="181"/>
+      <c r="C53" s="181"/>
+      <c r="D53" s="181"/>
+      <c r="E53" s="181"/>
+      <c r="F53" s="181"/>
+      <c r="G53" s="181"/>
+      <c r="H53" s="181"/>
+      <c r="I53" s="181"/>
+      <c r="J53" s="181"/>
+      <c r="K53" s="181"/>
+      <c r="L53" s="181"/>
+      <c r="M53" s="181"/>
+      <c r="N53" s="181"/>
+      <c r="O53" s="181"/>
+      <c r="P53" s="181"/>
+      <c r="Q53" s="181"/>
+      <c r="R53" s="181"/>
+      <c r="S53" s="181"/>
+      <c r="T53" s="181"/>
+      <c r="U53" s="181"/>
+      <c r="V53" s="181"/>
+      <c r="W53" s="181"/>
+      <c r="X53" s="181"/>
+      <c r="Y53" s="181"/>
+      <c r="Z53" s="181"/>
+      <c r="AA53" s="181"/>
+      <c r="AB53" s="181"/>
+      <c r="AC53" s="181"/>
+      <c r="AD53" s="181"/>
+      <c r="AE53" s="181"/>
+      <c r="AF53" s="181"/>
+      <c r="AG53" s="181"/>
     </row>
     <row r="54" spans="1:36" ht="18" customHeight="1">
       <c r="A54" s="182" t="s">
         <v>235</v>
       </c>
-      <c r="B54" s="180"/>
-      <c r="C54" s="180"/>
-      <c r="D54" s="180"/>
-      <c r="E54" s="180"/>
-      <c r="F54" s="180"/>
-      <c r="G54" s="180"/>
-      <c r="H54" s="180"/>
-      <c r="I54" s="180"/>
-      <c r="J54" s="180"/>
-      <c r="K54" s="180"/>
-      <c r="L54" s="180"/>
-      <c r="M54" s="180"/>
-      <c r="N54" s="180"/>
-      <c r="O54" s="180"/>
-      <c r="P54" s="180"/>
-      <c r="Q54" s="180"/>
-      <c r="R54" s="180"/>
-      <c r="S54" s="180"/>
-      <c r="T54" s="180"/>
-      <c r="U54" s="180"/>
-      <c r="V54" s="180"/>
-      <c r="W54" s="180"/>
-      <c r="X54" s="180"/>
-      <c r="Y54" s="180"/>
-      <c r="Z54" s="180"/>
-      <c r="AA54" s="180"/>
-      <c r="AB54" s="180"/>
-      <c r="AC54" s="180"/>
-      <c r="AD54" s="180"/>
-      <c r="AE54" s="180"/>
-      <c r="AF54" s="180"/>
-      <c r="AG54" s="180"/>
+      <c r="B54" s="181"/>
+      <c r="C54" s="181"/>
+      <c r="D54" s="181"/>
+      <c r="E54" s="181"/>
+      <c r="F54" s="181"/>
+      <c r="G54" s="181"/>
+      <c r="H54" s="181"/>
+      <c r="I54" s="181"/>
+      <c r="J54" s="181"/>
+      <c r="K54" s="181"/>
+      <c r="L54" s="181"/>
+      <c r="M54" s="181"/>
+      <c r="N54" s="181"/>
+      <c r="O54" s="181"/>
+      <c r="P54" s="181"/>
+      <c r="Q54" s="181"/>
+      <c r="R54" s="181"/>
+      <c r="S54" s="181"/>
+      <c r="T54" s="181"/>
+      <c r="U54" s="181"/>
+      <c r="V54" s="181"/>
+      <c r="W54" s="181"/>
+      <c r="X54" s="181"/>
+      <c r="Y54" s="181"/>
+      <c r="Z54" s="181"/>
+      <c r="AA54" s="181"/>
+      <c r="AB54" s="181"/>
+      <c r="AC54" s="181"/>
+      <c r="AD54" s="181"/>
+      <c r="AE54" s="181"/>
+      <c r="AF54" s="181"/>
+      <c r="AG54" s="181"/>
     </row>
     <row r="55" spans="1:36" ht="22" customHeight="1">
       <c r="A55" s="149" t="s">
@@ -7421,36 +7420,36 @@
     </row>
     <row r="59" spans="1:36" ht="20.149999999999999" customHeight="1"/>
     <row r="60" spans="1:36" ht="24" customHeight="1">
-      <c r="A60" s="181" t="s">
+      <c r="A60" s="180" t="s">
         <v>236</v>
       </c>
-      <c r="B60" s="180"/>
-      <c r="C60" s="180"/>
-      <c r="D60" s="180"/>
-      <c r="E60" s="180"/>
-      <c r="F60" s="180"/>
-      <c r="G60" s="180"/>
-      <c r="H60" s="180"/>
-      <c r="I60" s="180"/>
-      <c r="J60" s="180"/>
-      <c r="K60" s="180"/>
-      <c r="L60" s="180"/>
+      <c r="B60" s="181"/>
+      <c r="C60" s="181"/>
+      <c r="D60" s="181"/>
+      <c r="E60" s="181"/>
+      <c r="F60" s="181"/>
+      <c r="G60" s="181"/>
+      <c r="H60" s="181"/>
+      <c r="I60" s="181"/>
+      <c r="J60" s="181"/>
+      <c r="K60" s="181"/>
+      <c r="L60" s="181"/>
     </row>
     <row r="61" spans="1:36" ht="20.149999999999999" customHeight="1">
       <c r="A61" s="182" t="s">
         <v>211</v>
       </c>
-      <c r="B61" s="180"/>
-      <c r="C61" s="180"/>
-      <c r="D61" s="180"/>
-      <c r="E61" s="180"/>
-      <c r="F61" s="180"/>
-      <c r="G61" s="180"/>
-      <c r="H61" s="180"/>
-      <c r="I61" s="180"/>
-      <c r="J61" s="180"/>
-      <c r="K61" s="180"/>
-      <c r="L61" s="180"/>
+      <c r="B61" s="181"/>
+      <c r="C61" s="181"/>
+      <c r="D61" s="181"/>
+      <c r="E61" s="181"/>
+      <c r="F61" s="181"/>
+      <c r="G61" s="181"/>
+      <c r="H61" s="181"/>
+      <c r="I61" s="181"/>
+      <c r="J61" s="181"/>
+      <c r="K61" s="181"/>
+      <c r="L61" s="181"/>
     </row>
     <row r="62" spans="1:36" ht="38.15" customHeight="1">
       <c r="A62" s="171" t="s">
@@ -7857,19 +7856,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:108" s="39" customFormat="1" ht="18">
-      <c r="A1" s="210" t="s">
+      <c r="A1" s="188" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="210"/>
-      <c r="C1" s="210"/>
-      <c r="D1" s="210"/>
-      <c r="E1" s="210"/>
-      <c r="F1" s="210"/>
-      <c r="G1" s="210"/>
-      <c r="H1" s="210"/>
-      <c r="I1" s="210"/>
-      <c r="J1" s="210"/>
-      <c r="K1" s="210"/>
+      <c r="B1" s="188"/>
+      <c r="C1" s="188"/>
+      <c r="D1" s="188"/>
+      <c r="E1" s="188"/>
+      <c r="F1" s="188"/>
+      <c r="G1" s="188"/>
+      <c r="H1" s="188"/>
+      <c r="I1" s="188"/>
+      <c r="J1" s="188"/>
+      <c r="K1" s="188"/>
       <c r="M1" s="3" t="s">
         <v>67</v>
       </c>
@@ -7999,12 +7998,12 @@
     </row>
     <row r="4" spans="1:108" s="39" customFormat="1" ht="14.25" customHeight="1">
       <c r="D4" s="43"/>
-      <c r="L4" s="211" t="s">
+      <c r="L4" s="189" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:108" ht="14.9" customHeight="1">
-      <c r="L5" s="212"/>
+      <c r="L5" s="190"/>
     </row>
     <row r="6" spans="1:108" s="39" customFormat="1" ht="14.25" customHeight="1">
       <c r="H6" s="44"/>
@@ -8036,23 +8035,23 @@
       <c r="B7" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="206" t="s">
+      <c r="C7" s="191" t="s">
         <v>72</v>
       </c>
-      <c r="D7" s="206"/>
-      <c r="E7" s="206"/>
-      <c r="F7" s="206"/>
-      <c r="G7" s="206"/>
-      <c r="H7" s="206"/>
-      <c r="I7" s="206"/>
-      <c r="J7" s="206"/>
-      <c r="K7" s="206"/>
-      <c r="L7" s="206"/>
-      <c r="M7" s="206"/>
-      <c r="N7" s="206"/>
-      <c r="O7" s="206"/>
-      <c r="P7" s="206"/>
-      <c r="Q7" s="206"/>
+      <c r="D7" s="191"/>
+      <c r="E7" s="191"/>
+      <c r="F7" s="191"/>
+      <c r="G7" s="191"/>
+      <c r="H7" s="191"/>
+      <c r="I7" s="191"/>
+      <c r="J7" s="191"/>
+      <c r="K7" s="191"/>
+      <c r="L7" s="191"/>
+      <c r="M7" s="191"/>
+      <c r="N7" s="191"/>
+      <c r="O7" s="191"/>
+      <c r="P7" s="191"/>
+      <c r="Q7" s="191"/>
       <c r="R7" s="49"/>
       <c r="S7" s="49"/>
       <c r="T7" s="49"/>
@@ -8070,43 +8069,43 @@
     </row>
     <row r="9" spans="1:108" s="39" customFormat="1" ht="14.25" customHeight="1" thickBot="1">
       <c r="A9"/>
-      <c r="B9" s="213" t="s">
+      <c r="B9" s="192" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="214" t="s">
+      <c r="D9" s="193" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="215"/>
-      <c r="F9" s="216"/>
-      <c r="G9" s="217">
+      <c r="E9" s="194"/>
+      <c r="F9" s="195"/>
+      <c r="G9" s="196">
         <v>2022</v>
       </c>
-      <c r="H9" s="218"/>
-      <c r="I9" s="218"/>
-      <c r="J9" s="218"/>
-      <c r="K9" s="180"/>
-      <c r="L9" s="180"/>
+      <c r="H9" s="197"/>
+      <c r="I9" s="197"/>
+      <c r="J9" s="197"/>
+      <c r="K9" s="181"/>
+      <c r="L9" s="181"/>
     </row>
     <row r="10" spans="1:108" s="39" customFormat="1" ht="14.25" customHeight="1" thickBot="1">
-      <c r="B10" s="213"/>
+      <c r="B10" s="192"/>
       <c r="D10" s="52" t="s">
         <v>144</v>
       </c>
       <c r="J10" s="51"/>
     </row>
     <row r="11" spans="1:108" s="39" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B11" s="213"/>
-      <c r="D11" s="219" t="s">
+      <c r="B11" s="192"/>
+      <c r="D11" s="198" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="220"/>
-      <c r="F11" s="220"/>
-      <c r="G11" s="220"/>
-      <c r="H11" s="220"/>
-      <c r="I11" s="220"/>
-      <c r="J11" s="220"/>
-      <c r="K11" s="220"/>
-      <c r="L11" s="220"/>
+      <c r="E11" s="199"/>
+      <c r="F11" s="199"/>
+      <c r="G11" s="199"/>
+      <c r="H11" s="199"/>
+      <c r="I11" s="199"/>
+      <c r="J11" s="199"/>
+      <c r="K11" s="199"/>
+      <c r="L11" s="199"/>
       <c r="W11" s="53"/>
       <c r="X11" s="54"/>
       <c r="Y11" s="54"/>
@@ -8114,18 +8113,18 @@
       <c r="AA11" s="54"/>
     </row>
     <row r="12" spans="1:108" s="39" customFormat="1" ht="17.25" customHeight="1" thickBot="1">
-      <c r="B12" s="213"/>
-      <c r="D12" s="221" t="s">
+      <c r="B12" s="192"/>
+      <c r="D12" s="200" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="222"/>
-      <c r="F12" s="222"/>
-      <c r="G12" s="222"/>
-      <c r="H12" s="222"/>
-      <c r="I12" s="222"/>
-      <c r="J12" s="222"/>
-      <c r="K12" s="222"/>
-      <c r="L12" s="223"/>
+      <c r="E12" s="201"/>
+      <c r="F12" s="201"/>
+      <c r="G12" s="201"/>
+      <c r="H12" s="201"/>
+      <c r="I12" s="201"/>
+      <c r="J12" s="201"/>
+      <c r="K12" s="201"/>
+      <c r="L12" s="202"/>
       <c r="M12" s="55"/>
       <c r="W12" s="53"/>
       <c r="X12" s="54"/>
@@ -8134,16 +8133,16 @@
       <c r="AA12" s="54"/>
     </row>
     <row r="13" spans="1:108" s="39" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B13" s="213"/>
-      <c r="D13" s="224"/>
-      <c r="E13" s="225"/>
-      <c r="F13" s="225"/>
-      <c r="G13" s="225"/>
-      <c r="H13" s="225"/>
-      <c r="I13" s="225"/>
-      <c r="J13" s="225"/>
-      <c r="K13" s="225"/>
-      <c r="L13" s="226"/>
+      <c r="B13" s="192"/>
+      <c r="D13" s="203"/>
+      <c r="E13" s="204"/>
+      <c r="F13" s="204"/>
+      <c r="G13" s="204"/>
+      <c r="H13" s="204"/>
+      <c r="I13" s="204"/>
+      <c r="J13" s="204"/>
+      <c r="K13" s="204"/>
+      <c r="L13" s="205"/>
       <c r="W13" s="53"/>
       <c r="X13" s="54"/>
       <c r="Y13" s="54"/>
@@ -8151,49 +8150,49 @@
       <c r="AA13" s="54"/>
     </row>
     <row r="14" spans="1:108" ht="37.4" customHeight="1">
-      <c r="B14" s="213"/>
+      <c r="B14" s="192"/>
     </row>
     <row r="15" spans="1:108" ht="15" customHeight="1">
-      <c r="B15" s="213"/>
-      <c r="C15" s="227" t="s">
+      <c r="B15" s="192"/>
+      <c r="C15" s="206" t="s">
         <v>145</v>
       </c>
-      <c r="D15" s="227"/>
-      <c r="E15" s="227"/>
-      <c r="F15" s="227"/>
-      <c r="G15" s="227"/>
-      <c r="H15" s="227"/>
-      <c r="I15" s="227"/>
-      <c r="J15" s="227"/>
-      <c r="K15" s="227"/>
-      <c r="L15" s="227"/>
-      <c r="M15" s="227"/>
-      <c r="N15" s="227"/>
-      <c r="O15" s="227"/>
-      <c r="P15" s="227"/>
+      <c r="D15" s="206"/>
+      <c r="E15" s="206"/>
+      <c r="F15" s="206"/>
+      <c r="G15" s="206"/>
+      <c r="H15" s="206"/>
+      <c r="I15" s="206"/>
+      <c r="J15" s="206"/>
+      <c r="K15" s="206"/>
+      <c r="L15" s="206"/>
+      <c r="M15" s="206"/>
+      <c r="N15" s="206"/>
+      <c r="O15" s="206"/>
+      <c r="P15" s="206"/>
       <c r="Q15" s="56"/>
     </row>
     <row r="16" spans="1:108">
-      <c r="B16" s="213"/>
-      <c r="C16" s="227"/>
-      <c r="D16" s="227"/>
-      <c r="E16" s="227"/>
-      <c r="F16" s="227"/>
-      <c r="G16" s="227"/>
-      <c r="H16" s="227"/>
-      <c r="I16" s="227"/>
-      <c r="J16" s="227"/>
-      <c r="K16" s="227"/>
-      <c r="L16" s="227"/>
-      <c r="M16" s="227"/>
-      <c r="N16" s="227"/>
-      <c r="O16" s="227"/>
-      <c r="P16" s="227"/>
+      <c r="B16" s="192"/>
+      <c r="C16" s="206"/>
+      <c r="D16" s="206"/>
+      <c r="E16" s="206"/>
+      <c r="F16" s="206"/>
+      <c r="G16" s="206"/>
+      <c r="H16" s="206"/>
+      <c r="I16" s="206"/>
+      <c r="J16" s="206"/>
+      <c r="K16" s="206"/>
+      <c r="L16" s="206"/>
+      <c r="M16" s="206"/>
+      <c r="N16" s="206"/>
+      <c r="O16" s="206"/>
+      <c r="P16" s="206"/>
     </row>
     <row r="17" spans="2:39" ht="15" customHeight="1">
-      <c r="B17" s="213"/>
+      <c r="B17" s="192"/>
       <c r="C17" s="57"/>
-      <c r="D17" s="203" t="s">
+      <c r="D17" s="213" t="s">
         <v>77</v>
       </c>
       <c r="E17" s="1" t="s">
@@ -8201,9 +8200,9 @@
       </c>
     </row>
     <row r="18" spans="2:39" ht="15" customHeight="1">
-      <c r="B18" s="213"/>
+      <c r="B18" s="192"/>
       <c r="C18" s="57"/>
-      <c r="D18" s="204"/>
+      <c r="D18" s="214"/>
       <c r="F18" s="1" t="s">
         <v>143</v>
       </c>
@@ -8296,9 +8295,9 @@
       </c>
     </row>
     <row r="19" spans="2:39" ht="15" customHeight="1">
-      <c r="B19" s="213"/>
+      <c r="B19" s="192"/>
       <c r="C19" s="57"/>
-      <c r="D19" s="204"/>
+      <c r="D19" s="214"/>
       <c r="E19" t="s">
         <v>79</v>
       </c>
@@ -8394,9 +8393,9 @@
       </c>
     </row>
     <row r="20" spans="2:39" ht="15" customHeight="1">
-      <c r="B20" s="213"/>
+      <c r="B20" s="192"/>
       <c r="C20" s="57"/>
-      <c r="D20" s="205"/>
+      <c r="D20" s="215"/>
       <c r="E20" t="s">
         <v>80</v>
       </c>
@@ -8492,9 +8491,9 @@
       </c>
     </row>
     <row r="21" spans="2:39" ht="15" customHeight="1">
-      <c r="B21" s="213"/>
+      <c r="B21" s="192"/>
       <c r="C21" s="57"/>
-      <c r="D21" s="205"/>
+      <c r="D21" s="215"/>
       <c r="E21" t="s">
         <v>81</v>
       </c>
@@ -8590,9 +8589,9 @@
       </c>
     </row>
     <row r="22" spans="2:39" ht="15" customHeight="1">
-      <c r="B22" s="213"/>
+      <c r="B22" s="192"/>
       <c r="C22" s="57"/>
-      <c r="D22" s="205"/>
+      <c r="D22" s="215"/>
       <c r="F22" s="59"/>
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
@@ -8625,18 +8624,18 @@
       <c r="AI22" s="5"/>
     </row>
     <row r="23" spans="2:39" ht="15" customHeight="1">
-      <c r="B23" s="213"/>
+      <c r="B23" s="192"/>
       <c r="C23" s="57"/>
-      <c r="D23" s="205"/>
+      <c r="D23" s="215"/>
       <c r="E23" s="1" t="s">
         <v>82</v>
       </c>
       <c r="F23" s="59"/>
     </row>
     <row r="24" spans="2:39" ht="15" customHeight="1">
-      <c r="B24" s="213"/>
+      <c r="B24" s="192"/>
       <c r="C24" s="57"/>
-      <c r="D24" s="205"/>
+      <c r="D24" s="215"/>
       <c r="F24" s="1" t="s">
         <v>143</v>
       </c>
@@ -8729,9 +8728,9 @@
       </c>
     </row>
     <row r="25" spans="2:39" ht="15" customHeight="1">
-      <c r="B25" s="213"/>
+      <c r="B25" s="192"/>
       <c r="C25" s="57"/>
-      <c r="D25" s="205"/>
+      <c r="D25" s="215"/>
       <c r="E25" t="s">
         <v>79</v>
       </c>
@@ -8827,9 +8826,9 @@
       </c>
     </row>
     <row r="26" spans="2:39" ht="15" customHeight="1">
-      <c r="B26" s="213"/>
+      <c r="B26" s="192"/>
       <c r="C26" s="57"/>
-      <c r="D26" s="205"/>
+      <c r="D26" s="215"/>
       <c r="E26" t="s">
         <v>80</v>
       </c>
@@ -8925,9 +8924,9 @@
       </c>
     </row>
     <row r="27" spans="2:39" ht="15" customHeight="1">
-      <c r="B27" s="213"/>
+      <c r="B27" s="192"/>
       <c r="C27" s="57"/>
-      <c r="D27" s="205"/>
+      <c r="D27" s="215"/>
       <c r="E27" t="s">
         <v>81</v>
       </c>
@@ -9023,7 +9022,7 @@
       </c>
     </row>
     <row r="28" spans="2:39" ht="15" customHeight="1">
-      <c r="B28" s="213"/>
+      <c r="B28" s="192"/>
       <c r="C28" s="57"/>
       <c r="D28" s="57"/>
       <c r="G28" s="5"/>
@@ -9061,7 +9060,7 @@
       <c r="AM28" s="5"/>
     </row>
     <row r="29" spans="2:39" ht="15" customHeight="1">
-      <c r="B29" s="213"/>
+      <c r="B29" s="192"/>
       <c r="C29" s="57"/>
       <c r="D29" s="57"/>
       <c r="E29" s="1" t="s">
@@ -9103,7 +9102,7 @@
       <c r="AM29" s="5"/>
     </row>
     <row r="30" spans="2:39" ht="15" customHeight="1" thickBot="1">
-      <c r="B30" s="213"/>
+      <c r="B30" s="192"/>
       <c r="C30" s="57"/>
       <c r="D30" s="57"/>
       <c r="E30" s="1"/>
@@ -9143,9 +9142,9 @@
       <c r="AM30" s="5"/>
     </row>
     <row r="31" spans="2:39" ht="15" customHeight="1" thickBot="1">
-      <c r="B31" s="213"/>
+      <c r="B31" s="192"/>
       <c r="C31" s="57"/>
-      <c r="D31" s="204" t="s">
+      <c r="D31" s="214" t="s">
         <v>84</v>
       </c>
       <c r="E31" s="60" t="s">
@@ -9195,9 +9194,9 @@
       <c r="AM31" s="5"/>
     </row>
     <row r="32" spans="2:39" ht="15" customHeight="1">
-      <c r="B32" s="213"/>
+      <c r="B32" s="192"/>
       <c r="C32" s="57"/>
-      <c r="D32" s="204"/>
+      <c r="D32" s="214"/>
       <c r="E32" s="65" t="s">
         <v>90</v>
       </c>
@@ -9245,9 +9244,9 @@
       <c r="AM32" s="5"/>
     </row>
     <row r="33" spans="2:74" ht="15" customHeight="1">
-      <c r="B33" s="213"/>
+      <c r="B33" s="192"/>
       <c r="C33" s="57"/>
-      <c r="D33" s="204"/>
+      <c r="D33" s="214"/>
       <c r="E33" s="68" t="s">
         <v>95</v>
       </c>
@@ -9295,9 +9294,9 @@
       <c r="AM33" s="5"/>
     </row>
     <row r="34" spans="2:74" ht="15" customHeight="1">
-      <c r="B34" s="213"/>
+      <c r="B34" s="192"/>
       <c r="C34" s="57"/>
-      <c r="D34" s="204"/>
+      <c r="D34" s="214"/>
       <c r="E34" s="71" t="s">
         <v>97</v>
       </c>
@@ -9345,9 +9344,9 @@
       <c r="AM34" s="5"/>
     </row>
     <row r="35" spans="2:74" ht="15" customHeight="1">
-      <c r="B35" s="213"/>
+      <c r="B35" s="192"/>
       <c r="C35" s="57"/>
-      <c r="D35" s="204"/>
+      <c r="D35" s="214"/>
       <c r="E35" s="68" t="s">
         <v>99</v>
       </c>
@@ -9395,9 +9394,9 @@
       <c r="AM35" s="5"/>
     </row>
     <row r="36" spans="2:74" ht="15" customHeight="1" thickBot="1">
-      <c r="B36" s="213"/>
+      <c r="B36" s="192"/>
       <c r="C36" s="57"/>
-      <c r="D36" s="204"/>
+      <c r="D36" s="214"/>
       <c r="E36" s="74" t="s">
         <v>101</v>
       </c>
@@ -9484,23 +9483,23 @@
       <c r="AM37" s="5"/>
     </row>
     <row r="38" spans="2:74" s="39" customFormat="1" ht="14.25" customHeight="1">
-      <c r="C38" s="206" t="s">
+      <c r="C38" s="191" t="s">
         <v>103</v>
       </c>
-      <c r="D38" s="206"/>
-      <c r="E38" s="206"/>
-      <c r="F38" s="206"/>
-      <c r="G38" s="206"/>
-      <c r="H38" s="206"/>
-      <c r="I38" s="206"/>
-      <c r="J38" s="206"/>
-      <c r="K38" s="206"/>
-      <c r="L38" s="206"/>
-      <c r="M38" s="206"/>
-      <c r="N38" s="206"/>
-      <c r="O38" s="206"/>
-      <c r="P38" s="206"/>
-      <c r="Q38" s="206"/>
+      <c r="D38" s="191"/>
+      <c r="E38" s="191"/>
+      <c r="F38" s="191"/>
+      <c r="G38" s="191"/>
+      <c r="H38" s="191"/>
+      <c r="I38" s="191"/>
+      <c r="J38" s="191"/>
+      <c r="K38" s="191"/>
+      <c r="L38" s="191"/>
+      <c r="M38" s="191"/>
+      <c r="N38" s="191"/>
+      <c r="O38" s="191"/>
+      <c r="P38" s="191"/>
+      <c r="Q38" s="191"/>
       <c r="R38" s="49"/>
       <c r="S38" s="49"/>
       <c r="T38" s="49"/>
@@ -9633,10 +9632,10 @@
       </c>
     </row>
     <row r="43" spans="2:74" ht="15" customHeight="1">
-      <c r="B43" s="208" t="s">
+      <c r="B43" s="222" t="s">
         <v>60</v>
       </c>
-      <c r="D43" s="203" t="s">
+      <c r="D43" s="213" t="s">
         <v>105</v>
       </c>
       <c r="E43" s="78" t="s">
@@ -9738,8 +9737,8 @@
       </c>
     </row>
     <row r="44" spans="2:74">
-      <c r="B44" s="208"/>
-      <c r="D44" s="204"/>
+      <c r="B44" s="222"/>
+      <c r="D44" s="214"/>
       <c r="E44" s="81" t="s">
         <v>90</v>
       </c>
@@ -9839,8 +9838,8 @@
       </c>
     </row>
     <row r="45" spans="2:74">
-      <c r="B45" s="208"/>
-      <c r="D45" s="204"/>
+      <c r="B45" s="222"/>
+      <c r="D45" s="214"/>
       <c r="E45" s="82" t="s">
         <v>90</v>
       </c>
@@ -9940,8 +9939,8 @@
       </c>
     </row>
     <row r="46" spans="2:74">
-      <c r="B46" s="208"/>
-      <c r="D46" s="205"/>
+      <c r="B46" s="222"/>
+      <c r="D46" s="215"/>
       <c r="E46" s="78" t="s">
         <v>95</v>
       </c>
@@ -10074,8 +10073,8 @@
       <c r="BV46" s="5"/>
     </row>
     <row r="47" spans="2:74">
-      <c r="B47" s="208"/>
-      <c r="D47" s="205"/>
+      <c r="B47" s="222"/>
+      <c r="D47" s="215"/>
       <c r="E47" s="78" t="s">
         <v>95</v>
       </c>
@@ -10208,8 +10207,8 @@
       <c r="BV47" s="5"/>
     </row>
     <row r="48" spans="2:74">
-      <c r="B48" s="208"/>
-      <c r="D48" s="205"/>
+      <c r="B48" s="222"/>
+      <c r="D48" s="215"/>
       <c r="E48" s="78" t="s">
         <v>95</v>
       </c>
@@ -10342,8 +10341,8 @@
       <c r="BV48" s="5"/>
     </row>
     <row r="49" spans="2:74">
-      <c r="B49" s="208"/>
-      <c r="D49" s="205"/>
+      <c r="B49" s="222"/>
+      <c r="D49" s="215"/>
       <c r="E49" s="78" t="s">
         <v>97</v>
       </c>
@@ -10476,8 +10475,8 @@
       <c r="BV49" s="5"/>
     </row>
     <row r="50" spans="2:74">
-      <c r="B50" s="208"/>
-      <c r="D50" s="205"/>
+      <c r="B50" s="222"/>
+      <c r="D50" s="215"/>
       <c r="E50" s="78" t="s">
         <v>97</v>
       </c>
@@ -10610,8 +10609,8 @@
       <c r="BV50" s="5"/>
     </row>
     <row r="51" spans="2:74">
-      <c r="B51" s="208"/>
-      <c r="D51" s="205"/>
+      <c r="B51" s="222"/>
+      <c r="D51" s="215"/>
       <c r="E51" s="78" t="s">
         <v>97</v>
       </c>
@@ -10744,8 +10743,8 @@
       <c r="BV51" s="5"/>
     </row>
     <row r="52" spans="2:74">
-      <c r="B52" s="208"/>
-      <c r="D52" s="205"/>
+      <c r="B52" s="222"/>
+      <c r="D52" s="215"/>
       <c r="E52" s="78" t="s">
         <v>99</v>
       </c>
@@ -10878,8 +10877,8 @@
       <c r="BV52" s="5"/>
     </row>
     <row r="53" spans="2:74">
-      <c r="B53" s="208"/>
-      <c r="D53" s="205"/>
+      <c r="B53" s="222"/>
+      <c r="D53" s="215"/>
       <c r="E53" s="78" t="s">
         <v>99</v>
       </c>
@@ -11012,8 +11011,8 @@
       <c r="BV53" s="5"/>
     </row>
     <row r="54" spans="2:74">
-      <c r="B54" s="208"/>
-      <c r="D54" s="205"/>
+      <c r="B54" s="222"/>
+      <c r="D54" s="215"/>
       <c r="E54" s="78" t="s">
         <v>99</v>
       </c>
@@ -11146,8 +11145,8 @@
       <c r="BV54" s="5"/>
     </row>
     <row r="55" spans="2:74">
-      <c r="B55" s="208"/>
-      <c r="D55" s="205"/>
+      <c r="B55" s="222"/>
+      <c r="D55" s="215"/>
       <c r="E55" s="78" t="s">
         <v>101</v>
       </c>
@@ -11280,8 +11279,8 @@
       <c r="BV55" s="5"/>
     </row>
     <row r="56" spans="2:74">
-      <c r="B56" s="208"/>
-      <c r="D56" s="205"/>
+      <c r="B56" s="222"/>
+      <c r="D56" s="215"/>
       <c r="E56" s="78" t="s">
         <v>101</v>
       </c>
@@ -11414,8 +11413,8 @@
       <c r="BV56" s="5"/>
     </row>
     <row r="57" spans="2:74">
-      <c r="B57" s="208"/>
-      <c r="D57" s="205"/>
+      <c r="B57" s="222"/>
+      <c r="D57" s="215"/>
       <c r="E57" s="78" t="s">
         <v>101</v>
       </c>
@@ -11548,7 +11547,7 @@
       <c r="BV57" s="5"/>
     </row>
     <row r="58" spans="2:74">
-      <c r="B58" s="208"/>
+      <c r="B58" s="222"/>
       <c r="D58" s="57"/>
       <c r="E58" s="81"/>
       <c r="F58" s="81"/>
@@ -11617,7 +11616,7 @@
       <c r="BV58" s="5"/>
     </row>
     <row r="59" spans="2:74">
-      <c r="B59" s="208"/>
+      <c r="B59" s="222"/>
       <c r="D59" s="57"/>
       <c r="E59" s="81"/>
       <c r="F59" s="81"/>
@@ -11686,7 +11685,7 @@
       <c r="BV59" s="5"/>
     </row>
     <row r="60" spans="2:74">
-      <c r="B60" s="208"/>
+      <c r="B60" s="222"/>
       <c r="D60" s="57"/>
       <c r="E60" s="81"/>
       <c r="F60" s="81"/>
@@ -11755,7 +11754,7 @@
       <c r="BV60" s="5"/>
     </row>
     <row r="61" spans="2:74">
-      <c r="B61" s="208"/>
+      <c r="B61" s="222"/>
       <c r="D61" s="83"/>
       <c r="E61" s="81"/>
       <c r="F61" s="81"/>
@@ -11851,8 +11850,8 @@
       </c>
     </row>
     <row r="62" spans="2:74">
-      <c r="B62" s="208"/>
-      <c r="D62" s="203" t="s">
+      <c r="B62" s="222"/>
+      <c r="D62" s="213" t="s">
         <v>106</v>
       </c>
       <c r="E62" s="78" t="s">
@@ -11954,8 +11953,8 @@
       </c>
     </row>
     <row r="63" spans="2:74">
-      <c r="B63" s="208"/>
-      <c r="D63" s="204"/>
+      <c r="B63" s="222"/>
+      <c r="D63" s="214"/>
       <c r="E63" s="81" t="s">
         <v>90</v>
       </c>
@@ -12055,8 +12054,8 @@
       </c>
     </row>
     <row r="64" spans="2:74">
-      <c r="B64" s="208"/>
-      <c r="D64" s="204"/>
+      <c r="B64" s="222"/>
+      <c r="D64" s="214"/>
       <c r="E64" s="82" t="s">
         <v>90</v>
       </c>
@@ -12156,8 +12155,8 @@
       </c>
     </row>
     <row r="65" spans="2:74">
-      <c r="B65" s="208"/>
-      <c r="D65" s="205"/>
+      <c r="B65" s="222"/>
+      <c r="D65" s="215"/>
       <c r="E65" s="78" t="s">
         <v>95</v>
       </c>
@@ -12257,8 +12256,8 @@
       </c>
     </row>
     <row r="66" spans="2:74">
-      <c r="B66" s="208"/>
-      <c r="D66" s="205"/>
+      <c r="B66" s="222"/>
+      <c r="D66" s="215"/>
       <c r="E66" s="78" t="s">
         <v>95</v>
       </c>
@@ -12358,8 +12357,8 @@
       </c>
     </row>
     <row r="67" spans="2:74">
-      <c r="B67" s="208"/>
-      <c r="D67" s="205"/>
+      <c r="B67" s="222"/>
+      <c r="D67" s="215"/>
       <c r="E67" s="78" t="s">
         <v>95</v>
       </c>
@@ -12459,8 +12458,8 @@
       </c>
     </row>
     <row r="68" spans="2:74">
-      <c r="B68" s="208"/>
-      <c r="D68" s="205"/>
+      <c r="B68" s="222"/>
+      <c r="D68" s="215"/>
       <c r="E68" s="78" t="s">
         <v>97</v>
       </c>
@@ -12560,8 +12559,8 @@
       </c>
     </row>
     <row r="69" spans="2:74">
-      <c r="B69" s="208"/>
-      <c r="D69" s="205"/>
+      <c r="B69" s="222"/>
+      <c r="D69" s="215"/>
       <c r="E69" s="78" t="s">
         <v>97</v>
       </c>
@@ -12661,8 +12660,8 @@
       </c>
     </row>
     <row r="70" spans="2:74">
-      <c r="B70" s="208"/>
-      <c r="D70" s="205"/>
+      <c r="B70" s="222"/>
+      <c r="D70" s="215"/>
       <c r="E70" s="78" t="s">
         <v>97</v>
       </c>
@@ -12762,8 +12761,8 @@
       </c>
     </row>
     <row r="71" spans="2:74">
-      <c r="B71" s="208"/>
-      <c r="D71" s="205"/>
+      <c r="B71" s="222"/>
+      <c r="D71" s="215"/>
       <c r="E71" s="78" t="s">
         <v>99</v>
       </c>
@@ -12896,8 +12895,8 @@
       <c r="BV71" s="5"/>
     </row>
     <row r="72" spans="2:74">
-      <c r="B72" s="208"/>
-      <c r="D72" s="205"/>
+      <c r="B72" s="222"/>
+      <c r="D72" s="215"/>
       <c r="E72" s="78" t="s">
         <v>99</v>
       </c>
@@ -13030,8 +13029,8 @@
       <c r="BV72" s="5"/>
     </row>
     <row r="73" spans="2:74">
-      <c r="B73" s="208"/>
-      <c r="D73" s="205"/>
+      <c r="B73" s="222"/>
+      <c r="D73" s="215"/>
       <c r="E73" s="78" t="s">
         <v>99</v>
       </c>
@@ -13164,8 +13163,8 @@
       <c r="BV73" s="5"/>
     </row>
     <row r="74" spans="2:74">
-      <c r="B74" s="208"/>
-      <c r="D74" s="205"/>
+      <c r="B74" s="222"/>
+      <c r="D74" s="215"/>
       <c r="E74" s="78" t="s">
         <v>101</v>
       </c>
@@ -13298,8 +13297,8 @@
       <c r="BV74" s="5"/>
     </row>
     <row r="75" spans="2:74">
-      <c r="B75" s="208"/>
-      <c r="D75" s="205"/>
+      <c r="B75" s="222"/>
+      <c r="D75" s="215"/>
       <c r="E75" s="78" t="s">
         <v>101</v>
       </c>
@@ -13432,8 +13431,8 @@
       <c r="BV75" s="5"/>
     </row>
     <row r="76" spans="2:74">
-      <c r="B76" s="208"/>
-      <c r="D76" s="205"/>
+      <c r="B76" s="222"/>
+      <c r="D76" s="215"/>
       <c r="E76" s="78" t="s">
         <v>101</v>
       </c>
@@ -13566,13 +13565,13 @@
       <c r="BV76" s="5"/>
     </row>
     <row r="77" spans="2:74">
-      <c r="B77" s="208"/>
+      <c r="B77" s="222"/>
       <c r="D77" s="83"/>
       <c r="E77" s="81"/>
       <c r="F77" s="81"/>
     </row>
     <row r="78" spans="2:74">
-      <c r="B78" s="208"/>
+      <c r="B78" s="222"/>
       <c r="D78" s="39"/>
       <c r="E78" s="84"/>
       <c r="F78" s="84"/>
@@ -13668,8 +13667,8 @@
       </c>
     </row>
     <row r="79" spans="2:74">
-      <c r="B79" s="208"/>
-      <c r="D79" s="203" t="s">
+      <c r="B79" s="222"/>
+      <c r="D79" s="213" t="s">
         <v>107</v>
       </c>
       <c r="E79" s="78" t="s">
@@ -13771,8 +13770,8 @@
       <c r="AO79" s="1"/>
     </row>
     <row r="80" spans="2:74">
-      <c r="B80" s="208"/>
-      <c r="D80" s="204"/>
+      <c r="B80" s="222"/>
+      <c r="D80" s="214"/>
       <c r="E80" s="81" t="s">
         <v>90</v>
       </c>
@@ -13872,8 +13871,8 @@
       <c r="AO80" s="1"/>
     </row>
     <row r="81" spans="2:41">
-      <c r="B81" s="208"/>
-      <c r="D81" s="204"/>
+      <c r="B81" s="222"/>
+      <c r="D81" s="214"/>
       <c r="E81" s="82" t="s">
         <v>90</v>
       </c>
@@ -13973,8 +13972,8 @@
       <c r="AO81" s="1"/>
     </row>
     <row r="82" spans="2:41">
-      <c r="B82" s="209"/>
-      <c r="D82" s="205"/>
+      <c r="B82" s="223"/>
+      <c r="D82" s="215"/>
       <c r="E82" s="78" t="s">
         <v>95</v>
       </c>
@@ -14073,8 +14072,8 @@
       </c>
     </row>
     <row r="83" spans="2:41">
-      <c r="B83" s="209"/>
-      <c r="D83" s="205"/>
+      <c r="B83" s="223"/>
+      <c r="D83" s="215"/>
       <c r="E83" s="78" t="s">
         <v>95</v>
       </c>
@@ -14173,8 +14172,8 @@
       </c>
     </row>
     <row r="84" spans="2:41">
-      <c r="B84" s="209"/>
-      <c r="D84" s="205"/>
+      <c r="B84" s="223"/>
+      <c r="D84" s="215"/>
       <c r="E84" s="78" t="s">
         <v>95</v>
       </c>
@@ -14275,8 +14274,8 @@
       <c r="AL84" s="5"/>
     </row>
     <row r="85" spans="2:41">
-      <c r="B85" s="209"/>
-      <c r="D85" s="205"/>
+      <c r="B85" s="223"/>
+      <c r="D85" s="215"/>
       <c r="E85" s="78" t="s">
         <v>97</v>
       </c>
@@ -14377,8 +14376,8 @@
       <c r="AL85" s="5"/>
     </row>
     <row r="86" spans="2:41">
-      <c r="B86" s="209"/>
-      <c r="D86" s="205"/>
+      <c r="B86" s="223"/>
+      <c r="D86" s="215"/>
       <c r="E86" s="78" t="s">
         <v>97</v>
       </c>
@@ -14479,8 +14478,8 @@
       <c r="AL86" s="5"/>
     </row>
     <row r="87" spans="2:41">
-      <c r="B87" s="209"/>
-      <c r="D87" s="205"/>
+      <c r="B87" s="223"/>
+      <c r="D87" s="215"/>
       <c r="E87" s="78" t="s">
         <v>97</v>
       </c>
@@ -14581,8 +14580,8 @@
       <c r="AL87" s="5"/>
     </row>
     <row r="88" spans="2:41">
-      <c r="B88" s="209"/>
-      <c r="D88" s="205"/>
+      <c r="B88" s="223"/>
+      <c r="D88" s="215"/>
       <c r="E88" s="78" t="s">
         <v>99</v>
       </c>
@@ -14683,8 +14682,8 @@
       <c r="AL88" s="5"/>
     </row>
     <row r="89" spans="2:41">
-      <c r="B89" s="209"/>
-      <c r="D89" s="205"/>
+      <c r="B89" s="223"/>
+      <c r="D89" s="215"/>
       <c r="E89" s="78" t="s">
         <v>99</v>
       </c>
@@ -14785,8 +14784,8 @@
       <c r="AL89" s="5"/>
     </row>
     <row r="90" spans="2:41">
-      <c r="B90" s="209"/>
-      <c r="D90" s="205"/>
+      <c r="B90" s="223"/>
+      <c r="D90" s="215"/>
       <c r="E90" s="78" t="s">
         <v>99</v>
       </c>
@@ -14887,8 +14886,8 @@
       <c r="AL90" s="5"/>
     </row>
     <row r="91" spans="2:41">
-      <c r="B91" s="209"/>
-      <c r="D91" s="205"/>
+      <c r="B91" s="223"/>
+      <c r="D91" s="215"/>
       <c r="E91" s="78" t="s">
         <v>101</v>
       </c>
@@ -14989,8 +14988,8 @@
       <c r="AL91" s="5"/>
     </row>
     <row r="92" spans="2:41">
-      <c r="B92" s="209"/>
-      <c r="D92" s="205"/>
+      <c r="B92" s="223"/>
+      <c r="D92" s="215"/>
       <c r="E92" s="78" t="s">
         <v>101</v>
       </c>
@@ -15091,8 +15090,8 @@
       <c r="AL92" s="5"/>
     </row>
     <row r="93" spans="2:41">
-      <c r="B93" s="209"/>
-      <c r="D93" s="205"/>
+      <c r="B93" s="223"/>
+      <c r="D93" s="215"/>
       <c r="E93" s="78" t="s">
         <v>101</v>
       </c>
@@ -15193,10 +15192,10 @@
       <c r="AL93" s="5"/>
     </row>
     <row r="94" spans="2:41">
-      <c r="B94" s="209"/>
+      <c r="B94" s="223"/>
     </row>
     <row r="95" spans="2:41" ht="15" customHeight="1">
-      <c r="B95" s="209"/>
+      <c r="B95" s="223"/>
       <c r="G95" s="1" t="s">
         <v>143</v>
       </c>
@@ -15289,8 +15288,8 @@
       </c>
     </row>
     <row r="96" spans="2:41">
-      <c r="B96" s="209"/>
-      <c r="D96" s="203" t="s">
+      <c r="B96" s="223"/>
+      <c r="D96" s="213" t="s">
         <v>108</v>
       </c>
       <c r="E96" s="78" t="s">
@@ -15391,8 +15390,8 @@
       </c>
     </row>
     <row r="97" spans="2:36">
-      <c r="B97" s="209"/>
-      <c r="D97" s="204"/>
+      <c r="B97" s="223"/>
+      <c r="D97" s="214"/>
       <c r="E97" s="81" t="s">
         <v>90</v>
       </c>
@@ -15491,8 +15490,8 @@
       </c>
     </row>
     <row r="98" spans="2:36">
-      <c r="B98" s="209"/>
-      <c r="D98" s="204"/>
+      <c r="B98" s="223"/>
+      <c r="D98" s="214"/>
       <c r="E98" s="82" t="s">
         <v>90</v>
       </c>
@@ -15591,8 +15590,8 @@
       </c>
     </row>
     <row r="99" spans="2:36">
-      <c r="B99" s="209"/>
-      <c r="D99" s="205"/>
+      <c r="B99" s="223"/>
+      <c r="D99" s="215"/>
       <c r="E99" s="78" t="s">
         <v>95</v>
       </c>
@@ -15691,8 +15690,8 @@
       </c>
     </row>
     <row r="100" spans="2:36">
-      <c r="B100" s="209"/>
-      <c r="D100" s="205"/>
+      <c r="B100" s="223"/>
+      <c r="D100" s="215"/>
       <c r="E100" s="78" t="s">
         <v>95</v>
       </c>
@@ -15791,8 +15790,8 @@
       </c>
     </row>
     <row r="101" spans="2:36">
-      <c r="B101" s="209"/>
-      <c r="D101" s="205"/>
+      <c r="B101" s="223"/>
+      <c r="D101" s="215"/>
       <c r="E101" s="78" t="s">
         <v>95</v>
       </c>
@@ -15891,8 +15890,8 @@
       </c>
     </row>
     <row r="102" spans="2:36">
-      <c r="B102" s="209"/>
-      <c r="D102" s="205"/>
+      <c r="B102" s="223"/>
+      <c r="D102" s="215"/>
       <c r="E102" s="78" t="s">
         <v>97</v>
       </c>
@@ -15991,8 +15990,8 @@
       </c>
     </row>
     <row r="103" spans="2:36">
-      <c r="B103" s="209"/>
-      <c r="D103" s="205"/>
+      <c r="B103" s="223"/>
+      <c r="D103" s="215"/>
       <c r="E103" s="78" t="s">
         <v>97</v>
       </c>
@@ -16091,8 +16090,8 @@
       </c>
     </row>
     <row r="104" spans="2:36">
-      <c r="B104" s="209"/>
-      <c r="D104" s="205"/>
+      <c r="B104" s="223"/>
+      <c r="D104" s="215"/>
       <c r="E104" s="78" t="s">
         <v>97</v>
       </c>
@@ -16191,8 +16190,8 @@
       </c>
     </row>
     <row r="105" spans="2:36">
-      <c r="B105" s="209"/>
-      <c r="D105" s="205"/>
+      <c r="B105" s="223"/>
+      <c r="D105" s="215"/>
       <c r="E105" s="78" t="s">
         <v>99</v>
       </c>
@@ -16291,8 +16290,8 @@
       </c>
     </row>
     <row r="106" spans="2:36">
-      <c r="B106" s="209"/>
-      <c r="D106" s="205"/>
+      <c r="B106" s="223"/>
+      <c r="D106" s="215"/>
       <c r="E106" s="78" t="s">
         <v>99</v>
       </c>
@@ -16391,8 +16390,8 @@
       </c>
     </row>
     <row r="107" spans="2:36">
-      <c r="B107" s="209"/>
-      <c r="D107" s="205"/>
+      <c r="B107" s="223"/>
+      <c r="D107" s="215"/>
       <c r="E107" s="78" t="s">
         <v>99</v>
       </c>
@@ -16491,8 +16490,8 @@
       </c>
     </row>
     <row r="108" spans="2:36">
-      <c r="B108" s="209"/>
-      <c r="D108" s="205"/>
+      <c r="B108" s="223"/>
+      <c r="D108" s="215"/>
       <c r="E108" s="78" t="s">
         <v>101</v>
       </c>
@@ -16591,8 +16590,8 @@
       </c>
     </row>
     <row r="109" spans="2:36">
-      <c r="B109" s="209"/>
-      <c r="D109" s="205"/>
+      <c r="B109" s="223"/>
+      <c r="D109" s="215"/>
       <c r="E109" s="78" t="s">
         <v>101</v>
       </c>
@@ -16691,8 +16690,8 @@
       </c>
     </row>
     <row r="110" spans="2:36">
-      <c r="B110" s="209"/>
-      <c r="D110" s="205"/>
+      <c r="B110" s="223"/>
+      <c r="D110" s="215"/>
       <c r="E110" s="78" t="s">
         <v>101</v>
       </c>
@@ -16791,10 +16790,10 @@
       </c>
     </row>
     <row r="111" spans="2:36">
-      <c r="B111" s="209"/>
+      <c r="B111" s="223"/>
     </row>
     <row r="112" spans="2:36">
-      <c r="B112" s="209"/>
+      <c r="B112" s="223"/>
       <c r="G112" s="1" t="s">
         <v>143</v>
       </c>
@@ -16887,8 +16886,8 @@
       </c>
     </row>
     <row r="113" spans="2:36">
-      <c r="B113" s="209"/>
-      <c r="D113" s="203" t="s">
+      <c r="B113" s="223"/>
+      <c r="D113" s="213" t="s">
         <v>109</v>
       </c>
       <c r="E113" s="78" t="s">
@@ -16990,8 +16989,8 @@
       </c>
     </row>
     <row r="114" spans="2:36">
-      <c r="B114" s="209"/>
-      <c r="D114" s="204"/>
+      <c r="B114" s="223"/>
+      <c r="D114" s="214"/>
       <c r="E114" s="81" t="s">
         <v>90</v>
       </c>
@@ -17091,8 +17090,8 @@
       </c>
     </row>
     <row r="115" spans="2:36">
-      <c r="B115" s="209"/>
-      <c r="D115" s="204"/>
+      <c r="B115" s="223"/>
+      <c r="D115" s="214"/>
       <c r="E115" s="82" t="s">
         <v>90</v>
       </c>
@@ -17192,8 +17191,8 @@
       </c>
     </row>
     <row r="116" spans="2:36">
-      <c r="B116" s="209"/>
-      <c r="D116" s="205"/>
+      <c r="B116" s="223"/>
+      <c r="D116" s="215"/>
       <c r="E116" s="78" t="s">
         <v>95</v>
       </c>
@@ -17293,8 +17292,8 @@
       </c>
     </row>
     <row r="117" spans="2:36">
-      <c r="B117" s="209"/>
-      <c r="D117" s="205"/>
+      <c r="B117" s="223"/>
+      <c r="D117" s="215"/>
       <c r="E117" s="78" t="s">
         <v>95</v>
       </c>
@@ -17394,8 +17393,8 @@
       </c>
     </row>
     <row r="118" spans="2:36">
-      <c r="B118" s="209"/>
-      <c r="D118" s="205"/>
+      <c r="B118" s="223"/>
+      <c r="D118" s="215"/>
       <c r="E118" s="78" t="s">
         <v>95</v>
       </c>
@@ -17495,8 +17494,8 @@
       </c>
     </row>
     <row r="119" spans="2:36">
-      <c r="B119" s="209"/>
-      <c r="D119" s="205"/>
+      <c r="B119" s="223"/>
+      <c r="D119" s="215"/>
       <c r="E119" s="78" t="s">
         <v>97</v>
       </c>
@@ -17596,8 +17595,8 @@
       </c>
     </row>
     <row r="120" spans="2:36">
-      <c r="B120" s="209"/>
-      <c r="D120" s="205"/>
+      <c r="B120" s="223"/>
+      <c r="D120" s="215"/>
       <c r="E120" s="78" t="s">
         <v>97</v>
       </c>
@@ -17697,8 +17696,8 @@
       </c>
     </row>
     <row r="121" spans="2:36">
-      <c r="B121" s="209"/>
-      <c r="D121" s="205"/>
+      <c r="B121" s="223"/>
+      <c r="D121" s="215"/>
       <c r="E121" s="78" t="s">
         <v>97</v>
       </c>
@@ -17798,8 +17797,8 @@
       </c>
     </row>
     <row r="122" spans="2:36">
-      <c r="B122" s="209"/>
-      <c r="D122" s="205"/>
+      <c r="B122" s="223"/>
+      <c r="D122" s="215"/>
       <c r="E122" s="78" t="s">
         <v>99</v>
       </c>
@@ -17899,8 +17898,8 @@
       </c>
     </row>
     <row r="123" spans="2:36">
-      <c r="B123" s="209"/>
-      <c r="D123" s="205"/>
+      <c r="B123" s="223"/>
+      <c r="D123" s="215"/>
       <c r="E123" s="78" t="s">
         <v>99</v>
       </c>
@@ -18000,8 +17999,8 @@
       </c>
     </row>
     <row r="124" spans="2:36">
-      <c r="B124" s="209"/>
-      <c r="D124" s="205"/>
+      <c r="B124" s="223"/>
+      <c r="D124" s="215"/>
       <c r="E124" s="78" t="s">
         <v>99</v>
       </c>
@@ -18101,8 +18100,8 @@
       </c>
     </row>
     <row r="125" spans="2:36">
-      <c r="B125" s="209"/>
-      <c r="D125" s="205"/>
+      <c r="B125" s="223"/>
+      <c r="D125" s="215"/>
       <c r="E125" s="78" t="s">
         <v>101</v>
       </c>
@@ -18202,8 +18201,8 @@
       </c>
     </row>
     <row r="126" spans="2:36">
-      <c r="B126" s="209"/>
-      <c r="D126" s="205"/>
+      <c r="B126" s="223"/>
+      <c r="D126" s="215"/>
       <c r="E126" s="78" t="s">
         <v>101</v>
       </c>
@@ -18303,8 +18302,8 @@
       </c>
     </row>
     <row r="127" spans="2:36">
-      <c r="B127" s="209"/>
-      <c r="D127" s="205"/>
+      <c r="B127" s="223"/>
+      <c r="D127" s="215"/>
       <c r="E127" s="78" t="s">
         <v>101</v>
       </c>
@@ -18407,23 +18406,23 @@
       <c r="B128" s="86"/>
     </row>
     <row r="129" spans="2:28">
-      <c r="B129" s="207" t="s">
+      <c r="B129" s="216" t="s">
         <v>110</v>
       </c>
-      <c r="C129" s="206"/>
-      <c r="D129" s="206"/>
-      <c r="E129" s="206"/>
-      <c r="F129" s="206"/>
-      <c r="G129" s="206"/>
-      <c r="H129" s="206"/>
-      <c r="I129" s="206"/>
-      <c r="J129" s="206"/>
-      <c r="K129" s="206"/>
-      <c r="L129" s="206"/>
-      <c r="M129" s="206"/>
-      <c r="N129" s="206"/>
-      <c r="O129" s="206"/>
-      <c r="P129" s="206"/>
+      <c r="C129" s="191"/>
+      <c r="D129" s="191"/>
+      <c r="E129" s="191"/>
+      <c r="F129" s="191"/>
+      <c r="G129" s="191"/>
+      <c r="H129" s="191"/>
+      <c r="I129" s="191"/>
+      <c r="J129" s="191"/>
+      <c r="K129" s="191"/>
+      <c r="L129" s="191"/>
+      <c r="M129" s="191"/>
+      <c r="N129" s="191"/>
+      <c r="O129" s="191"/>
+      <c r="P129" s="191"/>
       <c r="Q129" s="49"/>
       <c r="R129" s="49"/>
       <c r="S129" s="49"/>
@@ -18458,21 +18457,21 @@
     </row>
     <row r="131" spans="2:28">
       <c r="B131" s="39"/>
-      <c r="C131" s="197" t="s">
+      <c r="C131" s="217" t="s">
         <v>111</v>
       </c>
-      <c r="D131" s="198"/>
-      <c r="E131" s="198"/>
-      <c r="F131" s="198"/>
-      <c r="G131" s="198"/>
-      <c r="H131" s="198"/>
-      <c r="I131" s="200" t="s">
+      <c r="D131" s="218"/>
+      <c r="E131" s="218"/>
+      <c r="F131" s="218"/>
+      <c r="G131" s="218"/>
+      <c r="H131" s="218"/>
+      <c r="I131" s="219" t="s">
         <v>112</v>
       </c>
-      <c r="J131" s="201"/>
-      <c r="K131" s="201"/>
-      <c r="L131" s="201"/>
-      <c r="M131" s="202"/>
+      <c r="J131" s="220"/>
+      <c r="K131" s="220"/>
+      <c r="L131" s="220"/>
+      <c r="M131" s="221"/>
       <c r="N131" s="88" t="s">
         <v>113</v>
       </c>
@@ -18490,14 +18489,14 @@
     </row>
     <row r="132" spans="2:28" ht="14.9" customHeight="1">
       <c r="B132" s="39"/>
-      <c r="C132" s="187" t="s">
+      <c r="C132" s="207" t="s">
         <v>115</v>
       </c>
-      <c r="D132" s="188"/>
-      <c r="E132" s="188"/>
-      <c r="F132" s="188"/>
-      <c r="G132" s="188"/>
-      <c r="H132" s="189"/>
+      <c r="D132" s="208"/>
+      <c r="E132" s="208"/>
+      <c r="F132" s="208"/>
+      <c r="G132" s="208"/>
+      <c r="H132" s="209"/>
       <c r="I132" t="s">
         <v>92</v>
       </c>
@@ -18508,14 +18507,14 @@
     </row>
     <row r="133" spans="2:28" ht="14.9" customHeight="1">
       <c r="B133" s="39"/>
-      <c r="C133" s="187" t="s">
+      <c r="C133" s="207" t="s">
         <v>116</v>
       </c>
-      <c r="D133" s="188"/>
-      <c r="E133" s="188"/>
-      <c r="F133" s="188"/>
-      <c r="G133" s="188"/>
-      <c r="H133" s="189"/>
+      <c r="D133" s="208"/>
+      <c r="E133" s="208"/>
+      <c r="F133" s="208"/>
+      <c r="G133" s="208"/>
+      <c r="H133" s="209"/>
       <c r="I133" s="99" t="s">
         <v>92</v>
       </c>
@@ -18538,21 +18537,21 @@
     </row>
     <row r="134" spans="2:28" ht="45" customHeight="1">
       <c r="B134" s="39"/>
-      <c r="C134" s="187" t="s">
+      <c r="C134" s="207" t="s">
         <v>105</v>
       </c>
-      <c r="D134" s="188"/>
-      <c r="E134" s="188"/>
-      <c r="F134" s="188"/>
-      <c r="G134" s="188"/>
-      <c r="H134" s="189"/>
-      <c r="I134" s="193" t="s">
+      <c r="D134" s="208"/>
+      <c r="E134" s="208"/>
+      <c r="F134" s="208"/>
+      <c r="G134" s="208"/>
+      <c r="H134" s="209"/>
+      <c r="I134" s="210" t="s">
         <v>118</v>
       </c>
-      <c r="J134" s="194"/>
-      <c r="K134" s="194"/>
-      <c r="L134" s="194"/>
-      <c r="M134" s="195"/>
+      <c r="J134" s="211"/>
+      <c r="K134" s="211"/>
+      <c r="L134" s="211"/>
+      <c r="M134" s="212"/>
       <c r="N134" s="104"/>
       <c r="O134" s="104"/>
       <c r="P134" s="105"/>
@@ -18566,21 +18565,21 @@
     </row>
     <row r="135" spans="2:28" ht="46.5" customHeight="1">
       <c r="B135" s="39"/>
-      <c r="C135" s="187" t="s">
+      <c r="C135" s="207" t="s">
         <v>119</v>
       </c>
-      <c r="D135" s="188"/>
-      <c r="E135" s="188"/>
-      <c r="F135" s="188"/>
-      <c r="G135" s="188"/>
-      <c r="H135" s="189"/>
-      <c r="I135" s="193" t="s">
+      <c r="D135" s="208"/>
+      <c r="E135" s="208"/>
+      <c r="F135" s="208"/>
+      <c r="G135" s="208"/>
+      <c r="H135" s="209"/>
+      <c r="I135" s="210" t="s">
         <v>120</v>
       </c>
-      <c r="J135" s="194"/>
-      <c r="K135" s="194"/>
-      <c r="L135" s="194"/>
-      <c r="M135" s="195"/>
+      <c r="J135" s="211"/>
+      <c r="K135" s="211"/>
+      <c r="L135" s="211"/>
+      <c r="M135" s="212"/>
       <c r="N135" s="104"/>
       <c r="O135" s="104"/>
       <c r="P135" s="105"/>
@@ -18594,14 +18593,14 @@
     </row>
     <row r="136" spans="2:28">
       <c r="B136" s="39"/>
-      <c r="C136" s="187" t="s">
+      <c r="C136" s="207" t="s">
         <v>121</v>
       </c>
-      <c r="D136" s="188"/>
-      <c r="E136" s="188"/>
-      <c r="F136" s="188"/>
-      <c r="G136" s="188"/>
-      <c r="H136" s="189"/>
+      <c r="D136" s="208"/>
+      <c r="E136" s="208"/>
+      <c r="F136" s="208"/>
+      <c r="G136" s="208"/>
+      <c r="H136" s="209"/>
       <c r="I136" s="107" t="s">
         <v>92</v>
       </c>
@@ -18622,14 +18621,14 @@
     </row>
     <row r="137" spans="2:28" ht="15" thickBot="1">
       <c r="B137" s="39"/>
-      <c r="C137" s="190" t="s">
+      <c r="C137" s="224" t="s">
         <v>122</v>
       </c>
-      <c r="D137" s="191"/>
-      <c r="E137" s="191"/>
-      <c r="F137" s="191"/>
-      <c r="G137" s="191"/>
-      <c r="H137" s="192"/>
+      <c r="D137" s="225"/>
+      <c r="E137" s="225"/>
+      <c r="F137" s="225"/>
+      <c r="G137" s="225"/>
+      <c r="H137" s="226"/>
       <c r="I137" s="111" t="s">
         <v>92</v>
       </c>
@@ -18650,12 +18649,12 @@
     </row>
     <row r="138" spans="2:28" ht="15" thickBot="1">
       <c r="B138" s="39"/>
-      <c r="C138" s="196"/>
-      <c r="D138" s="196"/>
-      <c r="E138" s="196"/>
-      <c r="F138" s="196"/>
-      <c r="G138" s="196"/>
-      <c r="H138" s="196"/>
+      <c r="C138" s="227"/>
+      <c r="D138" s="227"/>
+      <c r="E138" s="227"/>
+      <c r="F138" s="227"/>
+      <c r="G138" s="227"/>
+      <c r="H138" s="227"/>
       <c r="I138" s="115"/>
       <c r="J138" s="115"/>
       <c r="K138" s="115"/>
@@ -18674,21 +18673,21 @@
     </row>
     <row r="139" spans="2:28">
       <c r="B139" s="39"/>
-      <c r="C139" s="197" t="s">
+      <c r="C139" s="217" t="s">
         <v>123</v>
       </c>
-      <c r="D139" s="198"/>
-      <c r="E139" s="198"/>
-      <c r="F139" s="198"/>
-      <c r="G139" s="198"/>
-      <c r="H139" s="199"/>
-      <c r="I139" s="200" t="s">
+      <c r="D139" s="218"/>
+      <c r="E139" s="218"/>
+      <c r="F139" s="218"/>
+      <c r="G139" s="218"/>
+      <c r="H139" s="228"/>
+      <c r="I139" s="219" t="s">
         <v>112</v>
       </c>
-      <c r="J139" s="201"/>
-      <c r="K139" s="201"/>
-      <c r="L139" s="201"/>
-      <c r="M139" s="202"/>
+      <c r="J139" s="220"/>
+      <c r="K139" s="220"/>
+      <c r="L139" s="220"/>
+      <c r="M139" s="221"/>
       <c r="N139" s="88" t="s">
         <v>113</v>
       </c>
@@ -18706,14 +18705,14 @@
     </row>
     <row r="140" spans="2:28">
       <c r="B140" s="39"/>
-      <c r="C140" s="187" t="s">
+      <c r="C140" s="207" t="s">
         <v>116</v>
       </c>
-      <c r="D140" s="188"/>
-      <c r="E140" s="188"/>
-      <c r="F140" s="188"/>
-      <c r="G140" s="188"/>
-      <c r="H140" s="189"/>
+      <c r="D140" s="208"/>
+      <c r="E140" s="208"/>
+      <c r="F140" s="208"/>
+      <c r="G140" s="208"/>
+      <c r="H140" s="209"/>
       <c r="I140" s="99" t="s">
         <v>92</v>
       </c>
@@ -18797,14 +18796,14 @@
     </row>
     <row r="143" spans="2:28">
       <c r="B143" s="39"/>
-      <c r="C143" s="187" t="s">
+      <c r="C143" s="207" t="s">
         <v>119</v>
       </c>
-      <c r="D143" s="188"/>
-      <c r="E143" s="188"/>
-      <c r="F143" s="188"/>
-      <c r="G143" s="188"/>
-      <c r="H143" s="189"/>
+      <c r="D143" s="208"/>
+      <c r="E143" s="208"/>
+      <c r="F143" s="208"/>
+      <c r="G143" s="208"/>
+      <c r="H143" s="209"/>
       <c r="I143" s="121" t="s">
         <v>124</v>
       </c>
@@ -18825,14 +18824,14 @@
     </row>
     <row r="144" spans="2:28">
       <c r="B144" s="39"/>
-      <c r="C144" s="187" t="s">
+      <c r="C144" s="207" t="s">
         <v>121</v>
       </c>
-      <c r="D144" s="188"/>
-      <c r="E144" s="188"/>
-      <c r="F144" s="188"/>
-      <c r="G144" s="188"/>
-      <c r="H144" s="189"/>
+      <c r="D144" s="208"/>
+      <c r="E144" s="208"/>
+      <c r="F144" s="208"/>
+      <c r="G144" s="208"/>
+      <c r="H144" s="209"/>
       <c r="I144" s="121" t="s">
         <v>124</v>
       </c>
@@ -18853,14 +18852,14 @@
     </row>
     <row r="145" spans="2:23" ht="15" thickBot="1">
       <c r="B145" s="39"/>
-      <c r="C145" s="190" t="s">
+      <c r="C145" s="224" t="s">
         <v>127</v>
       </c>
-      <c r="D145" s="191"/>
-      <c r="E145" s="191"/>
-      <c r="F145" s="191"/>
-      <c r="G145" s="191"/>
-      <c r="H145" s="192"/>
+      <c r="D145" s="225"/>
+      <c r="E145" s="225"/>
+      <c r="F145" s="225"/>
+      <c r="G145" s="225"/>
+      <c r="H145" s="226"/>
       <c r="I145" s="111" t="s">
         <v>92</v>
       </c>
@@ -19112,16 +19111,17 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="C7:Q7"/>
-    <mergeCell ref="B9:B36"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:L9"/>
-    <mergeCell ref="D11:L11"/>
-    <mergeCell ref="D12:L12"/>
-    <mergeCell ref="D13:L13"/>
-    <mergeCell ref="C15:P16"/>
+    <mergeCell ref="C140:H140"/>
+    <mergeCell ref="C143:H143"/>
+    <mergeCell ref="C144:H144"/>
+    <mergeCell ref="C145:H145"/>
+    <mergeCell ref="C135:H135"/>
+    <mergeCell ref="I135:M135"/>
+    <mergeCell ref="C136:H136"/>
+    <mergeCell ref="C137:H137"/>
+    <mergeCell ref="C138:H138"/>
+    <mergeCell ref="C139:H139"/>
+    <mergeCell ref="I139:M139"/>
     <mergeCell ref="C134:H134"/>
     <mergeCell ref="I134:M134"/>
     <mergeCell ref="D17:D27"/>
@@ -19138,17 +19138,16 @@
     <mergeCell ref="D79:D93"/>
     <mergeCell ref="D96:D110"/>
     <mergeCell ref="D113:D127"/>
-    <mergeCell ref="I135:M135"/>
-    <mergeCell ref="C136:H136"/>
-    <mergeCell ref="C137:H137"/>
-    <mergeCell ref="C138:H138"/>
-    <mergeCell ref="C139:H139"/>
-    <mergeCell ref="I139:M139"/>
-    <mergeCell ref="C140:H140"/>
-    <mergeCell ref="C143:H143"/>
-    <mergeCell ref="C144:H144"/>
-    <mergeCell ref="C145:H145"/>
-    <mergeCell ref="C135:H135"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="C7:Q7"/>
+    <mergeCell ref="B9:B36"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:L9"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="D13:L13"/>
+    <mergeCell ref="C15:P16"/>
   </mergeCells>
   <phoneticPr fontId="22" type="noConversion"/>
   <hyperlinks>
@@ -19192,27 +19191,27 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="14"/>
-      <c r="B2" s="228" t="s">
+      <c r="B2" s="229" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="229"/>
-      <c r="D2" s="230"/>
+      <c r="C2" s="230"/>
+      <c r="D2" s="231"/>
       <c r="E2" s="38"/>
-      <c r="F2" s="228" t="s">
+      <c r="F2" s="229" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="229"/>
-      <c r="H2" s="230"/>
-      <c r="I2" s="228" t="s">
+      <c r="G2" s="230"/>
+      <c r="H2" s="231"/>
+      <c r="I2" s="229" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="229"/>
-      <c r="K2" s="230"/>
-      <c r="L2" s="228" t="s">
+      <c r="J2" s="230"/>
+      <c r="K2" s="231"/>
+      <c r="L2" s="229" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="229"/>
-      <c r="N2" s="230"/>
+      <c r="M2" s="230"/>
+      <c r="N2" s="231"/>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="17" t="s">
@@ -20835,268 +20834,266 @@
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="232" customWidth="1"/>
-    <col min="2" max="2" width="21.453125" style="232" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" style="232"/>
-    <col min="4" max="4" width="9.90625" style="232" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="232"/>
+    <col min="1" max="1" width="11.08984375" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="9.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="231" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="231" t="s">
+      <c r="A1" s="179" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="179" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="232">
+      <c r="A2">
         <v>2021</v>
       </c>
-      <c r="B2" s="232">
+      <c r="B2">
         <f>KEEI_계산과정!D56</f>
         <v>184566.95229970396</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="232">
+      <c r="A3">
         <v>2022</v>
       </c>
-      <c r="B3" s="232">
+      <c r="B3">
         <f>KEEI_계산과정!E56</f>
         <v>177348.23877434694</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="232">
+      <c r="A4">
         <v>2023</v>
       </c>
-      <c r="B4" s="232">
+      <c r="B4">
         <f>KEEI_계산과정!F56</f>
         <v>170129.52524898993</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="232">
+      <c r="A5">
         <v>2024</v>
       </c>
-      <c r="B5" s="232">
+      <c r="B5">
         <f>KEEI_계산과정!G56</f>
         <v>162910.81172363291</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="232">
+      <c r="A6">
         <v>2025</v>
       </c>
-      <c r="B6" s="232">
+      <c r="B6">
         <f>KEEI_계산과정!H56</f>
         <v>155692.09819827593</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="232">
+      <c r="A7">
         <v>2026</v>
       </c>
-      <c r="B7" s="232">
+      <c r="B7">
         <f>KEEI_계산과정!I56</f>
         <v>148473.38467291894</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="232">
+      <c r="A8">
         <v>2027</v>
       </c>
-      <c r="B8" s="232">
+      <c r="B8">
         <f>KEEI_계산과정!J56</f>
         <v>141254.67114756192</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="232">
+      <c r="A9">
         <v>2028</v>
       </c>
-      <c r="B9" s="232">
+      <c r="B9">
         <f>KEEI_계산과정!K56</f>
         <v>134035.95762220494</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="232">
+      <c r="A10">
         <v>2029</v>
       </c>
-      <c r="B10" s="232">
+      <c r="B10">
         <f>KEEI_계산과정!L56</f>
         <v>126817.24409684792</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="232">
+      <c r="A11">
         <v>2030</v>
       </c>
-      <c r="B11" s="232">
+      <c r="B11">
         <f>KEEI_계산과정!M56</f>
         <v>119598.53057149092</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="232">
+      <c r="A12">
         <v>2031</v>
       </c>
-      <c r="B12" s="232">
+      <c r="B12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="232">
+      <c r="A13">
         <v>2032</v>
       </c>
-      <c r="B13" s="232">
+      <c r="B13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="232">
+      <c r="A14">
         <v>2033</v>
       </c>
-      <c r="B14" s="232">
+      <c r="B14">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="232">
+      <c r="A15">
         <v>2034</v>
       </c>
-      <c r="B15" s="232">
+      <c r="B15">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="232">
+      <c r="A16">
         <v>2035</v>
       </c>
-      <c r="B16" s="232">
+      <c r="B16">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="232">
+      <c r="A17">
         <v>2036</v>
       </c>
-      <c r="B17" s="232">
+      <c r="B17">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="232">
+      <c r="A18">
         <v>2037</v>
       </c>
-      <c r="B18" s="232">
+      <c r="B18">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="232">
+      <c r="A19">
         <v>2038</v>
       </c>
-      <c r="B19" s="232">
+      <c r="B19">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="232">
+      <c r="A20">
         <v>2039</v>
       </c>
-      <c r="B20" s="232">
+      <c r="B20">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="232">
+      <c r="A21">
         <v>2040</v>
       </c>
-      <c r="B21" s="232">
+      <c r="B21">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="232">
+      <c r="A22">
         <v>2041</v>
       </c>
-      <c r="B22" s="232">
+      <c r="B22">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="232">
+      <c r="A23">
         <v>2042</v>
       </c>
-      <c r="B23" s="232">
+      <c r="B23">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="232">
+      <c r="A24">
         <v>2043</v>
       </c>
-      <c r="B24" s="232">
+      <c r="B24">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="232">
+      <c r="A25">
         <v>2044</v>
       </c>
-      <c r="B25" s="232">
+      <c r="B25">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="232">
+      <c r="A26">
         <v>2045</v>
       </c>
-      <c r="B26" s="232">
+      <c r="B26">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="232">
+      <c r="A27">
         <v>2046</v>
       </c>
-      <c r="B27" s="232">
+      <c r="B27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="232">
+      <c r="A28">
         <v>2047</v>
       </c>
-      <c r="B28" s="232">
+      <c r="B28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="232">
+      <c r="A29">
         <v>2048</v>
       </c>
-      <c r="B29" s="232">
+      <c r="B29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="232">
+      <c r="A30">
         <v>2049</v>
       </c>
-      <c r="B30" s="232">
+      <c r="B30">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="232">
+      <c r="A31">
         <v>2050</v>
       </c>
-      <c r="B31" s="232">
+      <c r="B31">
         <v>0</v>
       </c>
     </row>
@@ -21114,287 +21111,285 @@
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="232" customWidth="1"/>
-    <col min="2" max="2" width="21.453125" style="232" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" style="232"/>
-    <col min="4" max="4" width="9.90625" style="232" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="232"/>
+    <col min="1" max="1" width="11.08984375" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="9.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="231" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="231" t="s">
+      <c r="A1" s="179" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="179" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="232">
+      <c r="A2">
         <v>2021</v>
       </c>
-      <c r="B2" s="232">
+      <c r="B2">
         <f>KEEI_계산과정!D48</f>
         <v>136839.65777514293</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="232">
+      <c r="A3">
         <v>2022</v>
       </c>
-      <c r="B3" s="232">
+      <c r="B3">
         <f>KEEI_계산과정!E48</f>
         <v>133600.36519098651</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="232">
+      <c r="A4">
         <v>2023</v>
       </c>
-      <c r="B4" s="232">
+      <c r="B4">
         <f>KEEI_계산과정!F48</f>
         <v>130361.07260683009</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="232">
+      <c r="A5">
         <v>2024</v>
       </c>
-      <c r="B5" s="232">
+      <c r="B5">
         <f>KEEI_계산과정!G48</f>
         <v>127121.78002267367</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="232">
+      <c r="A6">
         <v>2025</v>
       </c>
-      <c r="B6" s="232">
+      <c r="B6">
         <f>KEEI_계산과정!H48</f>
         <v>123882.48743851724</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="232">
+      <c r="A7">
         <v>2026</v>
       </c>
-      <c r="B7" s="232">
+      <c r="B7">
         <f>KEEI_계산과정!I48</f>
         <v>120643.19485436082</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="232">
+      <c r="A8">
         <v>2027</v>
       </c>
-      <c r="B8" s="232">
+      <c r="B8">
         <f>KEEI_계산과정!J48</f>
         <v>117403.9022702044</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="232">
+      <c r="A9">
         <v>2028</v>
       </c>
-      <c r="B9" s="232">
+      <c r="B9">
         <f>KEEI_계산과정!K48</f>
         <v>114164.60968604797</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="232">
+      <c r="A10">
         <v>2029</v>
       </c>
-      <c r="B10" s="232">
+      <c r="B10">
         <f>KEEI_계산과정!L48</f>
         <v>110925.31710189156</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="232">
+      <c r="A11">
         <v>2030</v>
       </c>
-      <c r="B11" s="232">
+      <c r="B11">
         <f>KEEI_계산과정!M48</f>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="232">
+      <c r="A12">
         <v>2031</v>
       </c>
-      <c r="B12" s="232">
+      <c r="B12">
         <f>B11</f>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="232">
+      <c r="A13">
         <v>2032</v>
       </c>
-      <c r="B13" s="232">
+      <c r="B13">
         <f t="shared" ref="B13:B31" si="0">B12</f>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="232">
+      <c r="A14">
         <v>2033</v>
       </c>
-      <c r="B14" s="232">
+      <c r="B14">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="232">
+      <c r="A15">
         <v>2034</v>
       </c>
-      <c r="B15" s="232">
+      <c r="B15">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="232">
+      <c r="A16">
         <v>2035</v>
       </c>
-      <c r="B16" s="232">
+      <c r="B16">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="232">
+      <c r="A17">
         <v>2036</v>
       </c>
-      <c r="B17" s="232">
+      <c r="B17">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="232">
+      <c r="A18">
         <v>2037</v>
       </c>
-      <c r="B18" s="232">
+      <c r="B18">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="232">
+      <c r="A19">
         <v>2038</v>
       </c>
-      <c r="B19" s="232">
+      <c r="B19">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="232">
+      <c r="A20">
         <v>2039</v>
       </c>
-      <c r="B20" s="232">
+      <c r="B20">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="232">
+      <c r="A21">
         <v>2040</v>
       </c>
-      <c r="B21" s="232">
+      <c r="B21">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="232">
+      <c r="A22">
         <v>2041</v>
       </c>
-      <c r="B22" s="232">
+      <c r="B22">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="232">
+      <c r="A23">
         <v>2042</v>
       </c>
-      <c r="B23" s="232">
+      <c r="B23">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="232">
+      <c r="A24">
         <v>2043</v>
       </c>
-      <c r="B24" s="232">
+      <c r="B24">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="232">
+      <c r="A25">
         <v>2044</v>
       </c>
-      <c r="B25" s="232">
+      <c r="B25">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="232">
+      <c r="A26">
         <v>2045</v>
       </c>
-      <c r="B26" s="232">
+      <c r="B26">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="232">
+      <c r="A27">
         <v>2046</v>
       </c>
-      <c r="B27" s="232">
+      <c r="B27">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="232">
+      <c r="A28">
         <v>2047</v>
       </c>
-      <c r="B28" s="232">
+      <c r="B28">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="232">
+      <c r="A29">
         <v>2048</v>
       </c>
-      <c r="B29" s="232">
+      <c r="B29">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="232">
+      <c r="A30">
         <v>2049</v>
       </c>
-      <c r="B30" s="232">
+      <c r="B30">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="232">
+      <c r="A31">
         <v>2050</v>
       </c>
-      <c r="B31" s="232">
+      <c r="B31">
         <f t="shared" si="0"/>
         <v>107686.02451773513</v>
       </c>
@@ -21410,182 +21405,206 @@
   <sheetPr>
     <tabColor rgb="FF003399"/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.90625" style="232" customWidth="1"/>
-    <col min="2" max="16384" width="8.7265625" style="232"/>
+    <col min="1" max="1" width="19.90625" customWidth="1"/>
+    <col min="2" max="6" width="9.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28">
-      <c r="A1" s="232" t="s">
+    <row r="1" spans="1:32">
+      <c r="A1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="232">
+      <c r="B1">
+        <v>2020</v>
+      </c>
+      <c r="C1">
+        <v>2021</v>
+      </c>
+      <c r="D1">
+        <v>2022</v>
+      </c>
+      <c r="E1">
+        <v>2023</v>
+      </c>
+      <c r="F1">
         <v>2024</v>
       </c>
-      <c r="C1" s="232">
+      <c r="G1">
         <v>2025</v>
       </c>
-      <c r="D1" s="232">
+      <c r="H1">
         <v>2026</v>
       </c>
-      <c r="E1" s="232">
+      <c r="I1">
         <v>2027</v>
       </c>
-      <c r="F1" s="232">
+      <c r="J1">
         <v>2028</v>
       </c>
-      <c r="G1" s="232">
+      <c r="K1">
         <v>2029</v>
       </c>
-      <c r="H1" s="232">
+      <c r="L1">
         <v>2030</v>
       </c>
-      <c r="I1" s="232">
+      <c r="M1">
         <v>2031</v>
       </c>
-      <c r="J1" s="232">
+      <c r="N1">
         <v>2032</v>
       </c>
-      <c r="K1" s="232">
+      <c r="O1">
         <v>2033</v>
       </c>
-      <c r="L1" s="232">
+      <c r="P1">
         <v>2034</v>
       </c>
-      <c r="M1" s="232">
+      <c r="Q1">
         <v>2035</v>
       </c>
-      <c r="N1" s="232">
+      <c r="R1">
         <v>2036</v>
       </c>
-      <c r="O1" s="232">
+      <c r="S1">
         <v>2037</v>
       </c>
-      <c r="P1" s="232">
+      <c r="T1">
         <v>2038</v>
       </c>
-      <c r="Q1" s="232">
+      <c r="U1">
         <v>2039</v>
       </c>
-      <c r="R1" s="232">
+      <c r="V1">
         <v>2040</v>
       </c>
-      <c r="S1" s="232">
+      <c r="W1">
         <v>2041</v>
       </c>
-      <c r="T1" s="232">
+      <c r="X1">
         <v>2042</v>
       </c>
-      <c r="U1" s="232">
+      <c r="Y1">
         <v>2043</v>
       </c>
-      <c r="V1" s="232">
+      <c r="Z1">
         <v>2044</v>
       </c>
-      <c r="W1" s="232">
+      <c r="AA1">
         <v>2045</v>
       </c>
-      <c r="X1" s="232">
+      <c r="AB1">
         <v>2046</v>
       </c>
-      <c r="Y1" s="232">
+      <c r="AC1">
         <v>2047</v>
       </c>
-      <c r="Z1" s="232">
+      <c r="AD1">
         <v>2048</v>
       </c>
-      <c r="AA1" s="232">
+      <c r="AE1">
         <v>2049</v>
       </c>
-      <c r="AB1" s="232">
+      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28">
-      <c r="A2" s="232" t="s">
+    <row r="2" spans="1:32">
+      <c r="A2" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="232">
+      <c r="B2">
         <v>0.2</v>
       </c>
-      <c r="C2" s="232">
+      <c r="C2">
         <v>0.2</v>
       </c>
-      <c r="D2" s="232">
+      <c r="D2">
         <v>0.2</v>
       </c>
-      <c r="E2" s="232">
+      <c r="E2">
         <v>0.2</v>
       </c>
-      <c r="F2" s="232">
+      <c r="F2">
         <v>0.2</v>
       </c>
-      <c r="G2" s="232">
+      <c r="G2">
         <v>0.2</v>
       </c>
-      <c r="H2" s="232">
+      <c r="H2">
         <v>0.2</v>
       </c>
-      <c r="I2" s="232">
+      <c r="I2">
         <v>0.2</v>
       </c>
-      <c r="J2" s="232">
+      <c r="J2">
         <v>0.2</v>
       </c>
-      <c r="K2" s="232">
+      <c r="K2">
         <v>0.2</v>
       </c>
-      <c r="L2" s="232">
+      <c r="L2">
         <v>0.2</v>
       </c>
-      <c r="M2" s="232">
+      <c r="M2">
         <v>0.2</v>
       </c>
-      <c r="N2" s="232">
+      <c r="N2">
         <v>0.2</v>
       </c>
-      <c r="O2" s="232">
+      <c r="O2">
         <v>0.2</v>
       </c>
-      <c r="P2" s="232">
+      <c r="P2">
         <v>0.2</v>
       </c>
-      <c r="Q2" s="232">
+      <c r="Q2">
         <v>0.2</v>
       </c>
-      <c r="R2" s="232">
+      <c r="R2">
         <v>0.2</v>
       </c>
-      <c r="S2" s="232">
+      <c r="S2">
         <v>0.2</v>
       </c>
-      <c r="T2" s="232">
+      <c r="T2">
         <v>0.2</v>
       </c>
-      <c r="U2" s="232">
+      <c r="U2">
         <v>0.2</v>
       </c>
-      <c r="V2" s="232">
+      <c r="V2">
         <v>0.2</v>
       </c>
-      <c r="W2" s="232">
+      <c r="W2">
         <v>0.2</v>
       </c>
-      <c r="X2" s="232">
+      <c r="X2">
         <v>0.2</v>
       </c>
-      <c r="Y2" s="232">
+      <c r="Y2">
         <v>0.2</v>
       </c>
-      <c r="Z2" s="232">
+      <c r="Z2">
         <v>0.2</v>
       </c>
-      <c r="AA2" s="232">
+      <c r="AA2">
         <v>0.2</v>
       </c>
-      <c r="AB2" s="232">
+      <c r="AB2">
+        <v>0.2</v>
+      </c>
+      <c r="AC2">
+        <v>0.2</v>
+      </c>
+      <c r="AD2">
+        <v>0.2</v>
+      </c>
+      <c r="AE2">
+        <v>0.2</v>
+      </c>
+      <c r="AF2">
         <v>0.2</v>
       </c>
     </row>

</xml_diff>